<commit_message>
Fix: corregir No. de Documento a A9.I1.F2 en celda O2 todas las hojas
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -1828,9 +1828,9 @@
       <c r="N2" s="13" t="n"/>
       <c r="O2" s="74" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="45" t="n"/>
@@ -3245,9 +3245,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -4664,9 +4664,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -5899,9 +5899,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -7312,9 +7312,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -8547,9 +8547,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -9744,9 +9744,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -10942,9 +10942,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>
@@ -12139,9 +12139,9 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento    A3.I1.F2
-Revision:                    00
-Fecha:                         08/06/2026</t>
+          <t>No. de Documento             A9.I1.F2
+Revision:                                    00
+Fecha:                        08/06/2026</t>
         </is>
       </c>
       <c r="P2" s="22" t="n"/>

</xml_diff>

<commit_message>
Fix: Conversion O2 = A9.I1.F1 (Termoformado queda A9.I1.F2)
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -1828,7 +1828,7 @@
       <c r="N2" s="13" t="n"/>
       <c r="O2" s="74" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -3245,7 +3245,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -4664,7 +4664,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -5899,7 +5899,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -7312,7 +7312,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -8547,7 +8547,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -9744,7 +9744,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -10942,7 +10942,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>
@@ -12139,7 +12139,7 @@
       <c r="N2" s="23" t="n"/>
       <c r="O2" s="81" t="inlineStr">
         <is>
-          <t>No. de Documento             A9.I1.F2
+          <t>No. de Documento             A9.I1.F1
 Revision:                                    00
 Fecha:                        08/06/2026</t>
         </is>

</xml_diff>

<commit_message>
feat: Rotary Press - nuevo ítem 26 Verificación continuidad fusibles (row 34)
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -5870,7 +5870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Q39"/>
+  <dimension ref="A2:Q41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -6901,252 +6901,267 @@
       <c r="Q33" s="46" t="n"/>
     </row>
     <row r="34" ht="17.4" customHeight="1">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="21" t="inlineStr">
-        <is>
-          <t>CALENDARIO  DE  MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="C34" s="22" t="n"/>
+      <c r="B34" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="C34" s="25" t="inlineStr">
+        <is>
+          <t>Verificación de continuidad en fusibles</t>
+        </is>
+      </c>
       <c r="D34" s="22" t="n"/>
       <c r="E34" s="22" t="n"/>
       <c r="F34" s="22" t="n"/>
       <c r="G34" s="22" t="n"/>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="22" t="n"/>
-      <c r="J34" s="22" t="n"/>
-      <c r="K34" s="22" t="n"/>
-      <c r="L34" s="22" t="n"/>
-      <c r="M34" s="23" t="n"/>
-      <c r="N34" s="33" t="inlineStr">
-        <is>
-          <t>VOLTAJE ALIMENTACIÓN</t>
-        </is>
-      </c>
-      <c r="O34" s="22" t="n"/>
-      <c r="P34" s="22" t="n"/>
-      <c r="Q34" s="23" t="n"/>
     </row>
     <row r="35" ht="17.4" customHeight="1">
       <c r="A35" s="11" t="n"/>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>ENE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>FEB</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>ABR</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>MAY</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>JUN</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>JUL</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>AGO</t>
-        </is>
-      </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>SEP</t>
-        </is>
-      </c>
-      <c r="K35" s="5" t="inlineStr">
-        <is>
-          <t>OCT</t>
-        </is>
-      </c>
-      <c r="L35" s="5" t="inlineStr">
-        <is>
-          <t>NOV</t>
-        </is>
-      </c>
-      <c r="M35" s="5" t="inlineStr">
-        <is>
-          <t>DIC</t>
-        </is>
-      </c>
-      <c r="N35" s="6" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="O35" s="6" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="P35" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="Q35" s="6" t="inlineStr">
-        <is>
-          <t>VAC</t>
-        </is>
-      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>CALENDARIO  DE  MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="22" t="n"/>
+      <c r="G35" s="22" t="n"/>
+      <c r="H35" s="22" t="n"/>
+      <c r="I35" s="22" t="n"/>
+      <c r="J35" s="22" t="n"/>
+      <c r="K35" s="22" t="n"/>
+      <c r="L35" s="22" t="n"/>
+      <c r="M35" s="23" t="n"/>
+      <c r="N35" s="33" t="inlineStr">
+        <is>
+          <t>VOLTAJE ALIMENTACIÓN</t>
+        </is>
+      </c>
+      <c r="O35" s="22" t="n"/>
+      <c r="P35" s="22" t="n"/>
+      <c r="Q35" s="23" t="n"/>
     </row>
     <row r="36" ht="17.4" customHeight="1">
       <c r="A36" s="11" t="n"/>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M36" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="N36" s="6" t="n"/>
-      <c r="O36" s="6" t="n"/>
-      <c r="P36" s="6" t="n"/>
-      <c r="Q36" s="6" t="n"/>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>ENE</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>FEB</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>ABR</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>MAY</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>JUN</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>NOV</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>DIC</t>
+        </is>
+      </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="Q36" s="6" t="inlineStr">
+        <is>
+          <t>VAC</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="11" t="n"/>
-      <c r="B37" s="70" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="N37" s="6" t="n"/>
+      <c r="O37" s="6" t="n"/>
+      <c r="P37" s="6" t="n"/>
+      <c r="Q37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="14.4" customHeight="1">
+      <c r="A38" s="11" t="n"/>
+      <c r="B38" s="70" t="inlineStr">
         <is>
           <t xml:space="preserve">Realizo: </t>
         </is>
       </c>
-      <c r="C37" s="45" t="n"/>
-      <c r="D37" s="45" t="n"/>
-      <c r="E37" s="45" t="n"/>
-      <c r="F37" s="45" t="n"/>
-      <c r="G37" s="46" t="n"/>
-      <c r="H37" s="71" t="inlineStr">
+      <c r="C38" s="45" t="n"/>
+      <c r="D38" s="45" t="n"/>
+      <c r="E38" s="45" t="n"/>
+      <c r="F38" s="45" t="n"/>
+      <c r="G38" s="46" t="n"/>
+      <c r="H38" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>
       </c>
-      <c r="I37" s="75" t="n"/>
-      <c r="J37" s="75" t="n"/>
-      <c r="K37" s="72" t="inlineStr">
+      <c r="I38" s="75" t="n"/>
+      <c r="J38" s="75" t="n"/>
+      <c r="K38" s="72" t="inlineStr">
         <is>
           <t>Supervisor de Producción: 
 Firma: _____________________________</t>
         </is>
       </c>
-      <c r="L37" s="45" t="n"/>
-      <c r="M37" s="45" t="n"/>
-      <c r="N37" s="45" t="n"/>
-      <c r="O37" s="45" t="n"/>
-      <c r="P37" s="45" t="n"/>
-      <c r="Q37" s="46" t="n"/>
-    </row>
-    <row r="38" ht="14.4" customHeight="1">
-      <c r="B38" s="70" t="inlineStr">
+      <c r="L38" s="45" t="n"/>
+      <c r="M38" s="45" t="n"/>
+      <c r="N38" s="45" t="n"/>
+      <c r="O38" s="45" t="n"/>
+      <c r="P38" s="45" t="n"/>
+      <c r="Q38" s="46" t="n"/>
+    </row>
+    <row r="39" ht="14.4" customHeight="1">
+      <c r="B39" s="70" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
-      <c r="C38" s="76" t="n"/>
-      <c r="D38" s="76" t="n"/>
-      <c r="E38" s="76" t="n"/>
-      <c r="F38" s="76" t="n"/>
-      <c r="G38" s="77" t="n"/>
-      <c r="K38" s="70" t="inlineStr">
+      <c r="C39" s="76" t="n"/>
+      <c r="D39" s="76" t="n"/>
+      <c r="E39" s="76" t="n"/>
+      <c r="F39" s="76" t="n"/>
+      <c r="G39" s="77" t="n"/>
+      <c r="K39" s="70" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
-      <c r="L38" s="76" t="n"/>
-      <c r="M38" s="76" t="n"/>
-      <c r="N38" s="76" t="n"/>
-      <c r="O38" s="76" t="n"/>
-      <c r="P38" s="76" t="n"/>
-      <c r="Q38" s="77" t="n"/>
-    </row>
-    <row r="39" ht="14.4" customHeight="1">
-      <c r="B39" s="78" t="n"/>
-      <c r="C39" s="79" t="n"/>
-      <c r="D39" s="79" t="n"/>
-      <c r="E39" s="79" t="n"/>
-      <c r="F39" s="79" t="n"/>
-      <c r="G39" s="80" t="n"/>
-      <c r="K39" s="78" t="n"/>
-      <c r="L39" s="79" t="n"/>
-      <c r="M39" s="79" t="n"/>
-      <c r="N39" s="79" t="n"/>
-      <c r="O39" s="79" t="n"/>
-      <c r="P39" s="79" t="n"/>
-      <c r="Q39" s="80" t="n"/>
-    </row>
+      <c r="L39" s="76" t="n"/>
+      <c r="M39" s="76" t="n"/>
+      <c r="N39" s="76" t="n"/>
+      <c r="O39" s="76" t="n"/>
+      <c r="P39" s="76" t="n"/>
+      <c r="Q39" s="77" t="n"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="78" t="n"/>
+      <c r="C40" s="79" t="n"/>
+      <c r="D40" s="79" t="n"/>
+      <c r="E40" s="79" t="n"/>
+      <c r="F40" s="79" t="n"/>
+      <c r="G40" s="80" t="n"/>
+      <c r="K40" s="78" t="n"/>
+      <c r="L40" s="79" t="n"/>
+      <c r="M40" s="79" t="n"/>
+      <c r="N40" s="79" t="n"/>
+      <c r="O40" s="79" t="n"/>
+      <c r="P40" s="79" t="n"/>
+      <c r="Q40" s="80" t="n"/>
+    </row>
+    <row r="41"/>
   </sheetData>
   <mergeCells count="72">
     <mergeCell ref="C30:J30"/>

</xml_diff>

<commit_message>
fix: Rotary Press - corregir merge row34 fusibles; eliminar item10 Limpieza residuos
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -186,7 +186,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -449,11 +449,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -652,6 +672,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5870,7 +5892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Q41"/>
+  <dimension ref="A2:Q40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -6343,16 +6365,10 @@
       <c r="P16" s="22" t="n"/>
       <c r="Q16" s="23" t="n"/>
     </row>
-    <row r="17" ht="25.05" customHeight="1">
+    <row r="17" customHeight="1">
       <c r="A17" s="11" t="n"/>
-      <c r="B17" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C17" s="25" t="inlineStr">
-        <is>
-          <t>Limpieza de residuos de material en zonas de corte y transporte</t>
-        </is>
-      </c>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="25" t="n"/>
       <c r="D17" s="22" t="n"/>
       <c r="E17" s="22" t="n"/>
       <c r="F17" s="22" t="n"/>
@@ -6900,19 +6916,25 @@
       <c r="P33" s="45" t="n"/>
       <c r="Q33" s="46" t="n"/>
     </row>
-    <row r="34" ht="17.4" customHeight="1">
+    <row r="34" ht="25.05" customHeight="1">
       <c r="B34" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="C34" s="25" t="inlineStr">
-        <is>
-          <t>Verificación de continuidad en fusibles</t>
-        </is>
-      </c>
+      <c r="C34" s="25" t="n"/>
       <c r="D34" s="22" t="n"/>
       <c r="E34" s="22" t="n"/>
       <c r="F34" s="22" t="n"/>
       <c r="G34" s="22" t="n"/>
+      <c r="H34" s="22" t="n"/>
+      <c r="I34" s="22" t="n"/>
+      <c r="J34" s="22" t="n"/>
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="14" t="n"/>
+      <c r="M34" s="61" t="n"/>
+      <c r="N34" s="22" t="n"/>
+      <c r="O34" s="22" t="n"/>
+      <c r="P34" s="22" t="n"/>
+      <c r="Q34" s="23" t="n"/>
     </row>
     <row r="35" ht="17.4" customHeight="1">
       <c r="A35" s="11" t="n"/>
@@ -7031,65 +7053,29 @@
           <t>(   )</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="22" t="n"/>
+      <c r="F37" s="22" t="n"/>
+      <c r="G37" s="23" t="n"/>
       <c r="H37" s="4" t="inlineStr">
         <is>
           <t>(   )</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
+      <c r="I37" s="82" t="n"/>
+      <c r="J37" s="83" t="n"/>
       <c r="K37" s="4" t="inlineStr">
         <is>
           <t>(   )</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="N37" s="6" t="n"/>
-      <c r="O37" s="6" t="n"/>
-      <c r="P37" s="6" t="n"/>
-      <c r="Q37" s="6" t="n"/>
+      <c r="L37" s="22" t="n"/>
+      <c r="M37" s="22" t="n"/>
+      <c r="N37" s="22" t="n"/>
+      <c r="O37" s="22" t="n"/>
+      <c r="P37" s="22" t="n"/>
+      <c r="Q37" s="23" t="n"/>
     </row>
     <row r="38" ht="14.4" customHeight="1">
       <c r="A38" s="11" t="n"/>
@@ -7098,53 +7084,43 @@
           <t xml:space="preserve">Realizo: </t>
         </is>
       </c>
-      <c r="C38" s="45" t="n"/>
-      <c r="D38" s="45" t="n"/>
-      <c r="E38" s="45" t="n"/>
-      <c r="F38" s="45" t="n"/>
-      <c r="G38" s="46" t="n"/>
-      <c r="H38" s="71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha: </t>
-        </is>
-      </c>
-      <c r="I38" s="75" t="n"/>
-      <c r="J38" s="75" t="n"/>
+      <c r="C38" s="76" t="n"/>
+      <c r="D38" s="76" t="n"/>
+      <c r="E38" s="76" t="n"/>
+      <c r="F38" s="76" t="n"/>
+      <c r="G38" s="77" t="n"/>
+      <c r="H38" s="84" t="n"/>
+      <c r="J38" s="11" t="n"/>
       <c r="K38" s="72" t="inlineStr">
         <is>
           <t>Supervisor de Producción: 
 Firma: _____________________________</t>
         </is>
       </c>
-      <c r="L38" s="45" t="n"/>
-      <c r="M38" s="45" t="n"/>
-      <c r="N38" s="45" t="n"/>
-      <c r="O38" s="45" t="n"/>
-      <c r="P38" s="45" t="n"/>
-      <c r="Q38" s="46" t="n"/>
+      <c r="L38" s="76" t="n"/>
+      <c r="M38" s="76" t="n"/>
+      <c r="N38" s="76" t="n"/>
+      <c r="O38" s="76" t="n"/>
+      <c r="P38" s="76" t="n"/>
+      <c r="Q38" s="77" t="n"/>
     </row>
     <row r="39" ht="14.4" customHeight="1">
-      <c r="B39" s="70" t="inlineStr">
-        <is>
-          <t>Firma:</t>
-        </is>
-      </c>
-      <c r="C39" s="76" t="n"/>
-      <c r="D39" s="76" t="n"/>
-      <c r="E39" s="76" t="n"/>
-      <c r="F39" s="76" t="n"/>
-      <c r="G39" s="77" t="n"/>
-      <c r="K39" s="70" t="inlineStr">
-        <is>
-          <t>Firma:</t>
-        </is>
-      </c>
-      <c r="L39" s="76" t="n"/>
-      <c r="M39" s="76" t="n"/>
-      <c r="N39" s="76" t="n"/>
-      <c r="O39" s="76" t="n"/>
-      <c r="P39" s="76" t="n"/>
-      <c r="Q39" s="77" t="n"/>
+      <c r="B39" s="78" t="n"/>
+      <c r="C39" s="79" t="n"/>
+      <c r="D39" s="79" t="n"/>
+      <c r="E39" s="79" t="n"/>
+      <c r="F39" s="79" t="n"/>
+      <c r="G39" s="80" t="n"/>
+      <c r="H39" s="85" t="n"/>
+      <c r="I39" s="30" t="n"/>
+      <c r="J39" s="31" t="n"/>
+      <c r="K39" s="78" t="n"/>
+      <c r="L39" s="79" t="n"/>
+      <c r="M39" s="79" t="n"/>
+      <c r="N39" s="79" t="n"/>
+      <c r="O39" s="79" t="n"/>
+      <c r="P39" s="79" t="n"/>
+      <c r="Q39" s="80" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="78" t="n"/>
@@ -7161,19 +7137,18 @@
       <c r="P40" s="79" t="n"/>
       <c r="Q40" s="80" t="n"/>
     </row>
-    <row r="41"/>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="C34:J34"/>
+    <mergeCell ref="M34:Q34"/>
     <mergeCell ref="C30:J30"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C33:J33"/>
     <mergeCell ref="C24:J24"/>
     <mergeCell ref="J5:Q5"/>
-    <mergeCell ref="N34:Q34"/>
     <mergeCell ref="C14:J14"/>
     <mergeCell ref="M9:Q9"/>
     <mergeCell ref="K37:Q37"/>
-    <mergeCell ref="B34:M34"/>
     <mergeCell ref="C26:J26"/>
     <mergeCell ref="M20:Q20"/>
     <mergeCell ref="C29:J29"/>

</xml_diff>

<commit_message>
fix: restaurar formato Excel Rotary Press; ítem 10→fusibles row17; voltaje Entrada/Salida
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -186,7 +186,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -449,31 +449,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -672,8 +652,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5892,7 +5870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Q40"/>
+  <dimension ref="A2:Q39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -6365,10 +6343,16 @@
       <c r="P16" s="22" t="n"/>
       <c r="Q16" s="23" t="n"/>
     </row>
-    <row r="17" customHeight="1">
+    <row r="17" ht="25.05" customHeight="1">
       <c r="A17" s="11" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="25" t="n"/>
+      <c r="B17" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>Verificación de continuidad en fusibles</t>
+        </is>
+      </c>
       <c r="D17" s="22" t="n"/>
       <c r="E17" s="22" t="n"/>
       <c r="F17" s="22" t="n"/>
@@ -6916,11 +6900,14 @@
       <c r="P33" s="45" t="n"/>
       <c r="Q33" s="46" t="n"/>
     </row>
-    <row r="34" ht="25.05" customHeight="1">
-      <c r="B34" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="C34" s="25" t="n"/>
+    <row r="34" ht="17.4" customHeight="1">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>CALENDARIO  DE  MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="n"/>
       <c r="D34" s="22" t="n"/>
       <c r="E34" s="22" t="n"/>
       <c r="F34" s="22" t="n"/>
@@ -6928,160 +6915,212 @@
       <c r="H34" s="22" t="n"/>
       <c r="I34" s="22" t="n"/>
       <c r="J34" s="22" t="n"/>
-      <c r="K34" s="3" t="n"/>
-      <c r="L34" s="14" t="n"/>
-      <c r="M34" s="61" t="n"/>
-      <c r="N34" s="22" t="n"/>
+      <c r="K34" s="22" t="n"/>
+      <c r="L34" s="22" t="n"/>
+      <c r="M34" s="23" t="n"/>
+      <c r="N34" s="33" t="inlineStr">
+        <is>
+          <t>VOLTAJE ALIMENTACIÓN</t>
+        </is>
+      </c>
       <c r="O34" s="22" t="n"/>
       <c r="P34" s="22" t="n"/>
       <c r="Q34" s="23" t="n"/>
     </row>
     <row r="35" ht="17.4" customHeight="1">
       <c r="A35" s="11" t="n"/>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>CALENDARIO  DE  MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="C35" s="22" t="n"/>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="22" t="n"/>
-      <c r="F35" s="22" t="n"/>
-      <c r="G35" s="22" t="n"/>
-      <c r="H35" s="22" t="n"/>
-      <c r="I35" s="22" t="n"/>
-      <c r="J35" s="22" t="n"/>
-      <c r="K35" s="22" t="n"/>
-      <c r="L35" s="22" t="n"/>
-      <c r="M35" s="23" t="n"/>
-      <c r="N35" s="33" t="inlineStr">
-        <is>
-          <t>VOLTAJE ALIMENTACIÓN</t>
-        </is>
-      </c>
-      <c r="O35" s="22" t="n"/>
-      <c r="P35" s="22" t="n"/>
-      <c r="Q35" s="23" t="n"/>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>ENE</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>FEB</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>ABR</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>MAY</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>JUN</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>NOV</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>DIC</t>
+        </is>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="P35" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="Q35" s="6" t="inlineStr">
+        <is>
+          <t>VAC</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="17.4" customHeight="1">
       <c r="A36" s="11" t="n"/>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>ENE</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>FEB</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>ABR</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>MAY</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>JUN</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>JUL</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>AGO</t>
-        </is>
-      </c>
-      <c r="J36" s="5" t="inlineStr">
-        <is>
-          <t>SEP</t>
-        </is>
-      </c>
-      <c r="K36" s="5" t="inlineStr">
-        <is>
-          <t>OCT</t>
-        </is>
-      </c>
-      <c r="L36" s="5" t="inlineStr">
-        <is>
-          <t>NOV</t>
-        </is>
-      </c>
-      <c r="M36" s="5" t="inlineStr">
-        <is>
-          <t>DIC</t>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="O36" s="6" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="P36" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
-        </is>
-      </c>
+          <t>Entrada 220VAC</t>
+        </is>
+      </c>
+      <c r="O36" s="6" t="n"/>
+      <c r="P36" s="6" t="n"/>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>VAC</t>
+          <t>Salida 24VDC</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="11" t="n"/>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="C37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
-      <c r="E37" s="22" t="n"/>
-      <c r="F37" s="22" t="n"/>
-      <c r="G37" s="23" t="n"/>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="I37" s="82" t="n"/>
-      <c r="J37" s="83" t="n"/>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L37" s="22" t="n"/>
-      <c r="M37" s="22" t="n"/>
-      <c r="N37" s="22" t="n"/>
-      <c r="O37" s="22" t="n"/>
-      <c r="P37" s="22" t="n"/>
-      <c r="Q37" s="23" t="n"/>
+      <c r="B37" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Realizo: </t>
+        </is>
+      </c>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="46" t="n"/>
+      <c r="H37" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha: </t>
+        </is>
+      </c>
+      <c r="I37" s="75" t="n"/>
+      <c r="J37" s="75" t="n"/>
+      <c r="K37" s="72" t="inlineStr">
+        <is>
+          <t>Supervisor de Producción: 
+Firma: _____________________________</t>
+        </is>
+      </c>
+      <c r="L37" s="45" t="n"/>
+      <c r="M37" s="45" t="n"/>
+      <c r="N37" s="45" t="n"/>
+      <c r="O37" s="45" t="n"/>
+      <c r="P37" s="45" t="n"/>
+      <c r="Q37" s="46" t="n"/>
     </row>
     <row r="38" ht="14.4" customHeight="1">
-      <c r="A38" s="11" t="n"/>
       <c r="B38" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Realizo: </t>
+          <t>Firma:</t>
         </is>
       </c>
       <c r="C38" s="76" t="n"/>
@@ -7089,12 +7128,9 @@
       <c r="E38" s="76" t="n"/>
       <c r="F38" s="76" t="n"/>
       <c r="G38" s="77" t="n"/>
-      <c r="H38" s="84" t="n"/>
-      <c r="J38" s="11" t="n"/>
-      <c r="K38" s="72" t="inlineStr">
-        <is>
-          <t>Supervisor de Producción: 
-Firma: _____________________________</t>
+      <c r="K38" s="70" t="inlineStr">
+        <is>
+          <t>Firma:</t>
         </is>
       </c>
       <c r="L38" s="76" t="n"/>
@@ -7111,9 +7147,6 @@
       <c r="E39" s="79" t="n"/>
       <c r="F39" s="79" t="n"/>
       <c r="G39" s="80" t="n"/>
-      <c r="H39" s="85" t="n"/>
-      <c r="I39" s="30" t="n"/>
-      <c r="J39" s="31" t="n"/>
       <c r="K39" s="78" t="n"/>
       <c r="L39" s="79" t="n"/>
       <c r="M39" s="79" t="n"/>
@@ -7122,33 +7155,18 @@
       <c r="P39" s="79" t="n"/>
       <c r="Q39" s="80" t="n"/>
     </row>
-    <row r="40">
-      <c r="B40" s="78" t="n"/>
-      <c r="C40" s="79" t="n"/>
-      <c r="D40" s="79" t="n"/>
-      <c r="E40" s="79" t="n"/>
-      <c r="F40" s="79" t="n"/>
-      <c r="G40" s="80" t="n"/>
-      <c r="K40" s="78" t="n"/>
-      <c r="L40" s="79" t="n"/>
-      <c r="M40" s="79" t="n"/>
-      <c r="N40" s="79" t="n"/>
-      <c r="O40" s="79" t="n"/>
-      <c r="P40" s="79" t="n"/>
-      <c r="Q40" s="80" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="C34:J34"/>
-    <mergeCell ref="M34:Q34"/>
     <mergeCell ref="C30:J30"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C33:J33"/>
     <mergeCell ref="C24:J24"/>
     <mergeCell ref="J5:Q5"/>
+    <mergeCell ref="N34:Q34"/>
     <mergeCell ref="C14:J14"/>
     <mergeCell ref="M9:Q9"/>
     <mergeCell ref="K37:Q37"/>
+    <mergeCell ref="B34:M34"/>
     <mergeCell ref="C26:J26"/>
     <mergeCell ref="M20:Q20"/>
     <mergeCell ref="C29:J29"/>

</xml_diff>

<commit_message>
fix: Rotary Press voltaje Excel - Entrada 220VAC col14 / Salida 24VDC col15 juntos
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -7077,13 +7077,13 @@
           <t>Entrada 220VAC</t>
         </is>
       </c>
-      <c r="O36" s="6" t="n"/>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>Salida 24VDC</t>
+        </is>
+      </c>
       <c r="P36" s="6" t="n"/>
-      <c r="Q36" s="6" t="inlineStr">
-        <is>
-          <t>Salida 24VDC</t>
-        </is>
-      </c>
+      <c r="Q36" s="6" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="11" t="n"/>

</xml_diff>

<commit_message>
fix: Rotary Press voltaje headers - L1-L2 / VDC; borrar L3 y VAC
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -6991,24 +6991,16 @@
       </c>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L1-L2</t>
         </is>
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="P35" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="Q35" s="6" t="inlineStr">
-        <is>
-          <t>VAC</t>
-        </is>
-      </c>
+          <t>VDC</t>
+        </is>
+      </c>
+      <c r="P35" s="6" t="n"/>
+      <c r="Q35" s="6" t="n"/>
     </row>
     <row r="36" ht="17.4" customHeight="1">
       <c r="A36" s="11" t="n"/>
@@ -7072,16 +7064,8 @@
           <t>(   )</t>
         </is>
       </c>
-      <c r="N36" s="6" t="inlineStr">
-        <is>
-          <t>Entrada 220VAC</t>
-        </is>
-      </c>
-      <c r="O36" s="6" t="inlineStr">
-        <is>
-          <t>Salida 24VDC</t>
-        </is>
-      </c>
+      <c r="N36" s="6" t="n"/>
+      <c r="O36" s="6" t="n"/>
       <c r="P36" s="6" t="n"/>
       <c r="Q36" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix: Rotary Press quitar items 14 y 17 (rows 22/25); centrar fecha en Excel
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -453,7 +453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -652,6 +652,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6510,7 +6513,7 @@
       <c r="P21" s="22" t="n"/>
       <c r="Q21" s="23" t="n"/>
     </row>
-    <row r="22" ht="25.05" customHeight="1">
+    <row r="22" hidden="1" ht="25.05" customHeight="1">
       <c r="A22" s="11" t="n"/>
       <c r="B22" s="8" t="n">
         <v>14</v>
@@ -6609,7 +6612,7 @@
       <c r="P24" s="22" t="n"/>
       <c r="Q24" s="23" t="n"/>
     </row>
-    <row r="25" ht="25.05" customHeight="1">
+    <row r="25" hidden="1" ht="25.05" customHeight="1">
       <c r="A25" s="11" t="n"/>
       <c r="B25" s="8" t="n">
         <v>17</v>
@@ -7081,7 +7084,7 @@
       <c r="E37" s="45" t="n"/>
       <c r="F37" s="45" t="n"/>
       <c r="G37" s="46" t="n"/>
-      <c r="H37" s="71" t="inlineStr">
+      <c r="H37" s="84" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>

</xml_diff>

<commit_message>
Calender K1 Easy: VAC → Fuente 24VDC (rango 20-25V) en app y Excel
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -153,8 +153,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -234,8 +239,18 @@
         <fgColor rgb="00D6EAD8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001b5e20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002d8a45"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -512,11 +527,69 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -756,6 +829,17 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10980,7 +11064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N42"/>
+  <dimension ref="B1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11055,6 +11139,14 @@
           <t xml:space="preserve">  MECÁNICO</t>
         </is>
       </c>
+      <c r="C6" s="100" t="n"/>
+      <c r="D6" s="100" t="n"/>
+      <c r="E6" s="100" t="n"/>
+      <c r="F6" s="100" t="n"/>
+      <c r="G6" s="100" t="n"/>
+      <c r="H6" s="100" t="n"/>
+      <c r="I6" s="100" t="n"/>
+      <c r="J6" s="101" t="n"/>
       <c r="K6" s="87" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11070,6 +11162,7 @@
           <t>COMENTARIOS</t>
         </is>
       </c>
+      <c r="N6" s="101" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="88" t="inlineStr">
@@ -11082,6 +11175,13 @@
           <t>Inspección visual: ruidos, vibraciones y fugas en rodillos</t>
         </is>
       </c>
+      <c r="D7" s="100" t="n"/>
+      <c r="E7" s="100" t="n"/>
+      <c r="F7" s="100" t="n"/>
+      <c r="G7" s="100" t="n"/>
+      <c r="H7" s="100" t="n"/>
+      <c r="I7" s="100" t="n"/>
+      <c r="J7" s="101" t="n"/>
       <c r="K7" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11093,6 +11193,7 @@
         </is>
       </c>
       <c r="M7" s="91" t="n"/>
+      <c r="N7" s="101" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="92" t="inlineStr">
@@ -11105,6 +11206,13 @@
           <t>Lubricación de rodillos de calandria (baleros y chumaceras)</t>
         </is>
       </c>
+      <c r="D8" s="100" t="n"/>
+      <c r="E8" s="100" t="n"/>
+      <c r="F8" s="100" t="n"/>
+      <c r="G8" s="100" t="n"/>
+      <c r="H8" s="100" t="n"/>
+      <c r="I8" s="100" t="n"/>
+      <c r="J8" s="101" t="n"/>
       <c r="K8" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11116,6 +11224,7 @@
         </is>
       </c>
       <c r="M8" s="95" t="n"/>
+      <c r="N8" s="101" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="88" t="inlineStr">
@@ -11128,6 +11237,13 @@
           <t>Revisión y lubricación de cadena de transmisión y sprockets</t>
         </is>
       </c>
+      <c r="D9" s="100" t="n"/>
+      <c r="E9" s="100" t="n"/>
+      <c r="F9" s="100" t="n"/>
+      <c r="G9" s="100" t="n"/>
+      <c r="H9" s="100" t="n"/>
+      <c r="I9" s="100" t="n"/>
+      <c r="J9" s="101" t="n"/>
       <c r="K9" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11139,6 +11255,7 @@
         </is>
       </c>
       <c r="M9" s="91" t="n"/>
+      <c r="N9" s="101" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="92" t="inlineStr">
@@ -11151,6 +11268,13 @@
           <t>Verificación de tensión de cadena (deflexión máx. 1% de longitud)</t>
         </is>
       </c>
+      <c r="D10" s="100" t="n"/>
+      <c r="E10" s="100" t="n"/>
+      <c r="F10" s="100" t="n"/>
+      <c r="G10" s="100" t="n"/>
+      <c r="H10" s="100" t="n"/>
+      <c r="I10" s="100" t="n"/>
+      <c r="J10" s="101" t="n"/>
       <c r="K10" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11162,6 +11286,7 @@
         </is>
       </c>
       <c r="M10" s="95" t="n"/>
+      <c r="N10" s="101" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="88" t="inlineStr">
@@ -11174,6 +11299,13 @@
           <t>Revisión de caja reductora: nivel y calidad de aceite</t>
         </is>
       </c>
+      <c r="D11" s="100" t="n"/>
+      <c r="E11" s="100" t="n"/>
+      <c r="F11" s="100" t="n"/>
+      <c r="G11" s="100" t="n"/>
+      <c r="H11" s="100" t="n"/>
+      <c r="I11" s="100" t="n"/>
+      <c r="J11" s="101" t="n"/>
       <c r="K11" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11185,6 +11317,7 @@
         </is>
       </c>
       <c r="M11" s="91" t="n"/>
+      <c r="N11" s="101" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="92" t="inlineStr">
@@ -11197,6 +11330,13 @@
           <t>Verificación de alineación y paralelismo de rodillos</t>
         </is>
       </c>
+      <c r="D12" s="100" t="n"/>
+      <c r="E12" s="100" t="n"/>
+      <c r="F12" s="100" t="n"/>
+      <c r="G12" s="100" t="n"/>
+      <c r="H12" s="100" t="n"/>
+      <c r="I12" s="100" t="n"/>
+      <c r="J12" s="101" t="n"/>
       <c r="K12" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11208,6 +11348,7 @@
         </is>
       </c>
       <c r="M12" s="95" t="n"/>
+      <c r="N12" s="101" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="88" t="inlineStr">
@@ -11220,6 +11361,13 @@
           <t>Limpieza de rodillos y superficie de contacto (residuos de material)</t>
         </is>
       </c>
+      <c r="D13" s="100" t="n"/>
+      <c r="E13" s="100" t="n"/>
+      <c r="F13" s="100" t="n"/>
+      <c r="G13" s="100" t="n"/>
+      <c r="H13" s="100" t="n"/>
+      <c r="I13" s="100" t="n"/>
+      <c r="J13" s="101" t="n"/>
       <c r="K13" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11231,6 +11379,7 @@
         </is>
       </c>
       <c r="M13" s="91" t="n"/>
+      <c r="N13" s="101" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="92" t="inlineStr">
@@ -11243,6 +11392,13 @@
           <t>Revisión de tornillería y fijaciones estructurales</t>
         </is>
       </c>
+      <c r="D14" s="100" t="n"/>
+      <c r="E14" s="100" t="n"/>
+      <c r="F14" s="100" t="n"/>
+      <c r="G14" s="100" t="n"/>
+      <c r="H14" s="100" t="n"/>
+      <c r="I14" s="100" t="n"/>
+      <c r="J14" s="101" t="n"/>
       <c r="K14" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11254,6 +11410,7 @@
         </is>
       </c>
       <c r="M14" s="95" t="n"/>
+      <c r="N14" s="101" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="88" t="inlineStr">
@@ -11266,6 +11423,13 @@
           <t>Verificación del servo motor TECO JSMA-PSC44BK (temperatura y vibración)</t>
         </is>
       </c>
+      <c r="D15" s="100" t="n"/>
+      <c r="E15" s="100" t="n"/>
+      <c r="F15" s="100" t="n"/>
+      <c r="G15" s="100" t="n"/>
+      <c r="H15" s="100" t="n"/>
+      <c r="I15" s="100" t="n"/>
+      <c r="J15" s="101" t="n"/>
       <c r="K15" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11277,6 +11441,7 @@
         </is>
       </c>
       <c r="M15" s="91" t="n"/>
+      <c r="N15" s="101" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="86" t="inlineStr">
@@ -11284,6 +11449,14 @@
           <t xml:space="preserve">  ELÉCTRICO</t>
         </is>
       </c>
+      <c r="C16" s="100" t="n"/>
+      <c r="D16" s="100" t="n"/>
+      <c r="E16" s="100" t="n"/>
+      <c r="F16" s="100" t="n"/>
+      <c r="G16" s="100" t="n"/>
+      <c r="H16" s="100" t="n"/>
+      <c r="I16" s="100" t="n"/>
+      <c r="J16" s="101" t="n"/>
       <c r="K16" s="87" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11299,6 +11472,7 @@
           <t>COMENTARIOS</t>
         </is>
       </c>
+      <c r="N16" s="101" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="88" t="inlineStr">
@@ -11311,6 +11485,13 @@
           <t>Verificación del HMI MCU 01 TS: alarmas, indicadores y pantalla táctil</t>
         </is>
       </c>
+      <c r="D17" s="100" t="n"/>
+      <c r="E17" s="100" t="n"/>
+      <c r="F17" s="100" t="n"/>
+      <c r="G17" s="100" t="n"/>
+      <c r="H17" s="100" t="n"/>
+      <c r="I17" s="100" t="n"/>
+      <c r="J17" s="101" t="n"/>
       <c r="K17" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11322,6 +11503,7 @@
         </is>
       </c>
       <c r="M17" s="91" t="n"/>
+      <c r="N17" s="101" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="92" t="inlineStr">
@@ -11334,6 +11516,13 @@
           <t>Limpieza de tablero eléctrico y revisión de cableado y ducterías</t>
         </is>
       </c>
+      <c r="D18" s="100" t="n"/>
+      <c r="E18" s="100" t="n"/>
+      <c r="F18" s="100" t="n"/>
+      <c r="G18" s="100" t="n"/>
+      <c r="H18" s="100" t="n"/>
+      <c r="I18" s="100" t="n"/>
+      <c r="J18" s="101" t="n"/>
       <c r="K18" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11345,6 +11534,7 @@
         </is>
       </c>
       <c r="M18" s="95" t="n"/>
+      <c r="N18" s="101" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="88" t="inlineStr">
@@ -11357,6 +11547,13 @@
           <t>Reapriete de terminales y conexiones eléctricas</t>
         </is>
       </c>
+      <c r="D19" s="100" t="n"/>
+      <c r="E19" s="100" t="n"/>
+      <c r="F19" s="100" t="n"/>
+      <c r="G19" s="100" t="n"/>
+      <c r="H19" s="100" t="n"/>
+      <c r="I19" s="100" t="n"/>
+      <c r="J19" s="101" t="n"/>
       <c r="K19" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11368,6 +11565,7 @@
         </is>
       </c>
       <c r="M19" s="91" t="n"/>
+      <c r="N19" s="101" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="92" t="inlineStr">
@@ -11380,6 +11578,13 @@
           <t>Revisión de portafusibles Lovato FB01 B 2P: 2FU1, 6FU1, 7FU1</t>
         </is>
       </c>
+      <c r="D20" s="100" t="n"/>
+      <c r="E20" s="100" t="n"/>
+      <c r="F20" s="100" t="n"/>
+      <c r="G20" s="100" t="n"/>
+      <c r="H20" s="100" t="n"/>
+      <c r="I20" s="100" t="n"/>
+      <c r="J20" s="101" t="n"/>
       <c r="K20" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11391,6 +11596,7 @@
         </is>
       </c>
       <c r="M20" s="95" t="n"/>
+      <c r="N20" s="101" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="B21" s="88" t="inlineStr">
@@ -11403,6 +11609,13 @@
           <t>Verificación del relé de seguridad Allen-Bradley MSR126.1T (7K1)</t>
         </is>
       </c>
+      <c r="D21" s="100" t="n"/>
+      <c r="E21" s="100" t="n"/>
+      <c r="F21" s="100" t="n"/>
+      <c r="G21" s="100" t="n"/>
+      <c r="H21" s="100" t="n"/>
+      <c r="I21" s="100" t="n"/>
+      <c r="J21" s="101" t="n"/>
       <c r="K21" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11414,6 +11627,7 @@
         </is>
       </c>
       <c r="M21" s="91" t="n"/>
+      <c r="N21" s="101" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="B22" s="92" t="inlineStr">
@@ -11426,6 +11640,13 @@
           <t>Revisión del servo drive TECO: parámetros, fallas y conexiones</t>
         </is>
       </c>
+      <c r="D22" s="100" t="n"/>
+      <c r="E22" s="100" t="n"/>
+      <c r="F22" s="100" t="n"/>
+      <c r="G22" s="100" t="n"/>
+      <c r="H22" s="100" t="n"/>
+      <c r="I22" s="100" t="n"/>
+      <c r="J22" s="101" t="n"/>
       <c r="K22" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11437,6 +11658,7 @@
         </is>
       </c>
       <c r="M22" s="95" t="n"/>
+      <c r="N22" s="101" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="B23" s="88" t="inlineStr">
@@ -11449,6 +11671,13 @@
           <t>Verificación de fuente de poder Omron S8VK-C12024 (salida 24 VDC)</t>
         </is>
       </c>
+      <c r="D23" s="100" t="n"/>
+      <c r="E23" s="100" t="n"/>
+      <c r="F23" s="100" t="n"/>
+      <c r="G23" s="100" t="n"/>
+      <c r="H23" s="100" t="n"/>
+      <c r="I23" s="100" t="n"/>
+      <c r="J23" s="101" t="n"/>
       <c r="K23" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11460,6 +11689,7 @@
         </is>
       </c>
       <c r="M23" s="91" t="n"/>
+      <c r="N23" s="101" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="92" t="inlineStr">
@@ -11472,6 +11702,13 @@
           <t>Revisión del relevador SSR RM1A48D50 (7KPR1): temperatura y sujeción</t>
         </is>
       </c>
+      <c r="D24" s="100" t="n"/>
+      <c r="E24" s="100" t="n"/>
+      <c r="F24" s="100" t="n"/>
+      <c r="G24" s="100" t="n"/>
+      <c r="H24" s="100" t="n"/>
+      <c r="I24" s="100" t="n"/>
+      <c r="J24" s="101" t="n"/>
       <c r="K24" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11483,6 +11720,7 @@
         </is>
       </c>
       <c r="M24" s="95" t="n"/>
+      <c r="N24" s="101" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="88" t="inlineStr">
@@ -11495,6 +11733,13 @@
           <t>Prueba funcional: paro de emergencia y botón REAJUSTE EMERGENCIA</t>
         </is>
       </c>
+      <c r="D25" s="100" t="n"/>
+      <c r="E25" s="100" t="n"/>
+      <c r="F25" s="100" t="n"/>
+      <c r="G25" s="100" t="n"/>
+      <c r="H25" s="100" t="n"/>
+      <c r="I25" s="100" t="n"/>
+      <c r="J25" s="101" t="n"/>
       <c r="K25" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11506,6 +11751,7 @@
         </is>
       </c>
       <c r="M25" s="91" t="n"/>
+      <c r="N25" s="101" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="92" t="inlineStr">
@@ -11518,6 +11764,13 @@
           <t>Verificación de interruptor de seguridad Pizzato (funcionamiento y ajuste)</t>
         </is>
       </c>
+      <c r="D26" s="100" t="n"/>
+      <c r="E26" s="100" t="n"/>
+      <c r="F26" s="100" t="n"/>
+      <c r="G26" s="100" t="n"/>
+      <c r="H26" s="100" t="n"/>
+      <c r="I26" s="100" t="n"/>
+      <c r="J26" s="101" t="n"/>
       <c r="K26" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11529,6 +11782,7 @@
         </is>
       </c>
       <c r="M26" s="95" t="n"/>
+      <c r="N26" s="101" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="88" t="inlineStr">
@@ -11541,6 +11795,13 @@
           <t>Revisión del módulo I/O SHS DIN (señales de entrada/salida)</t>
         </is>
       </c>
+      <c r="D27" s="100" t="n"/>
+      <c r="E27" s="100" t="n"/>
+      <c r="F27" s="100" t="n"/>
+      <c r="G27" s="100" t="n"/>
+      <c r="H27" s="100" t="n"/>
+      <c r="I27" s="100" t="n"/>
+      <c r="J27" s="101" t="n"/>
       <c r="K27" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11552,6 +11813,7 @@
         </is>
       </c>
       <c r="M27" s="91" t="n"/>
+      <c r="N27" s="101" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="92" t="inlineStr">
@@ -11564,6 +11826,13 @@
           <t>Verificación del interruptor principal ABB OT25F4N2 (2QS1)</t>
         </is>
       </c>
+      <c r="D28" s="100" t="n"/>
+      <c r="E28" s="100" t="n"/>
+      <c r="F28" s="100" t="n"/>
+      <c r="G28" s="100" t="n"/>
+      <c r="H28" s="100" t="n"/>
+      <c r="I28" s="100" t="n"/>
+      <c r="J28" s="101" t="n"/>
       <c r="K28" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11575,6 +11844,7 @@
         </is>
       </c>
       <c r="M28" s="95" t="n"/>
+      <c r="N28" s="101" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="88" t="inlineStr">
@@ -11587,6 +11857,13 @@
           <t>Verificación de tierras físicas y continuidad de tierra</t>
         </is>
       </c>
+      <c r="D29" s="100" t="n"/>
+      <c r="E29" s="100" t="n"/>
+      <c r="F29" s="100" t="n"/>
+      <c r="G29" s="100" t="n"/>
+      <c r="H29" s="100" t="n"/>
+      <c r="I29" s="100" t="n"/>
+      <c r="J29" s="101" t="n"/>
       <c r="K29" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11598,6 +11875,7 @@
         </is>
       </c>
       <c r="M29" s="91" t="n"/>
+      <c r="N29" s="101" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="86" t="inlineStr">
@@ -11605,6 +11883,14 @@
           <t xml:space="preserve">  CALENTAMIENTO</t>
         </is>
       </c>
+      <c r="C30" s="100" t="n"/>
+      <c r="D30" s="100" t="n"/>
+      <c r="E30" s="100" t="n"/>
+      <c r="F30" s="100" t="n"/>
+      <c r="G30" s="100" t="n"/>
+      <c r="H30" s="100" t="n"/>
+      <c r="I30" s="100" t="n"/>
+      <c r="J30" s="101" t="n"/>
       <c r="K30" s="87" t="inlineStr">
         <is>
           <t>OK</t>
@@ -11620,6 +11906,7 @@
           <t>COMENTARIOS</t>
         </is>
       </c>
+      <c r="N30" s="101" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="88" t="inlineStr">
@@ -11632,6 +11919,13 @@
           <t>Verificación de temperatura de trabajo de rodillos calefactores</t>
         </is>
       </c>
+      <c r="D31" s="100" t="n"/>
+      <c r="E31" s="100" t="n"/>
+      <c r="F31" s="100" t="n"/>
+      <c r="G31" s="100" t="n"/>
+      <c r="H31" s="100" t="n"/>
+      <c r="I31" s="100" t="n"/>
+      <c r="J31" s="101" t="n"/>
       <c r="K31" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11643,6 +11937,7 @@
         </is>
       </c>
       <c r="M31" s="91" t="n"/>
+      <c r="N31" s="101" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="92" t="inlineStr">
@@ -11655,6 +11950,13 @@
           <t>Limpieza de resistencias calefactoras (polvo y residuos de material)</t>
         </is>
       </c>
+      <c r="D32" s="100" t="n"/>
+      <c r="E32" s="100" t="n"/>
+      <c r="F32" s="100" t="n"/>
+      <c r="G32" s="100" t="n"/>
+      <c r="H32" s="100" t="n"/>
+      <c r="I32" s="100" t="n"/>
+      <c r="J32" s="101" t="n"/>
       <c r="K32" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11666,6 +11968,7 @@
         </is>
       </c>
       <c r="M32" s="95" t="n"/>
+      <c r="N32" s="101" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="88" t="inlineStr">
@@ -11678,6 +11981,13 @@
           <t>Calibración de termocuplas y verificación de control de temperatura</t>
         </is>
       </c>
+      <c r="D33" s="100" t="n"/>
+      <c r="E33" s="100" t="n"/>
+      <c r="F33" s="100" t="n"/>
+      <c r="G33" s="100" t="n"/>
+      <c r="H33" s="100" t="n"/>
+      <c r="I33" s="100" t="n"/>
+      <c r="J33" s="101" t="n"/>
       <c r="K33" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11689,6 +11999,7 @@
         </is>
       </c>
       <c r="M33" s="91" t="n"/>
+      <c r="N33" s="101" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="92" t="inlineStr">
@@ -11701,6 +12012,13 @@
           <t>Medición eléctrica de resistencias calefactoras: continuidad y ohms</t>
         </is>
       </c>
+      <c r="D34" s="100" t="n"/>
+      <c r="E34" s="100" t="n"/>
+      <c r="F34" s="100" t="n"/>
+      <c r="G34" s="100" t="n"/>
+      <c r="H34" s="100" t="n"/>
+      <c r="I34" s="100" t="n"/>
+      <c r="J34" s="101" t="n"/>
       <c r="K34" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11712,6 +12030,7 @@
         </is>
       </c>
       <c r="M34" s="95" t="n"/>
+      <c r="N34" s="101" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="B35" s="88" t="inlineStr">
@@ -11724,6 +12043,13 @@
           <t>Verificación del SSR RM1A48D50 como control de calefacción (7KPR1)</t>
         </is>
       </c>
+      <c r="D35" s="100" t="n"/>
+      <c r="E35" s="100" t="n"/>
+      <c r="F35" s="100" t="n"/>
+      <c r="G35" s="100" t="n"/>
+      <c r="H35" s="100" t="n"/>
+      <c r="I35" s="100" t="n"/>
+      <c r="J35" s="101" t="n"/>
       <c r="K35" s="90" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11735,6 +12061,7 @@
         </is>
       </c>
       <c r="M35" s="91" t="n"/>
+      <c r="N35" s="101" t="n"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="B36" s="92" t="inlineStr">
@@ -11747,6 +12074,13 @@
           <t>Verificación de uniformidad de calor en todos los rodillos</t>
         </is>
       </c>
+      <c r="D36" s="100" t="n"/>
+      <c r="E36" s="100" t="n"/>
+      <c r="F36" s="100" t="n"/>
+      <c r="G36" s="100" t="n"/>
+      <c r="H36" s="100" t="n"/>
+      <c r="I36" s="100" t="n"/>
+      <c r="J36" s="101" t="n"/>
       <c r="K36" s="94" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -11758,6 +12092,7 @@
         </is>
       </c>
       <c r="M36" s="95" t="n"/>
+      <c r="N36" s="101" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="96" t="inlineStr">
@@ -11765,6 +12100,11 @@
           <t>CALENDARIO  DE  MANTENIMIENTO</t>
         </is>
       </c>
+      <c r="N37" s="102" t="inlineStr">
+        <is>
+          <t>VOLTAJE ALIMENTACIÓN</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="97" t="inlineStr">
@@ -11827,6 +12167,27 @@
           <t>DIC</t>
         </is>
       </c>
+      <c r="N38" s="103" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="O38" s="103" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="P38" s="103" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="Q38" s="103" t="inlineStr">
+        <is>
+          <t>Fuente 24VDC
+(20-25 V)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="94" t="inlineStr">
@@ -11889,6 +12250,10 @@
           <t>(   )</t>
         </is>
       </c>
+      <c r="N39" s="104" t="n"/>
+      <c r="O39" s="104" t="n"/>
+      <c r="P39" s="104" t="n"/>
+      <c r="Q39" s="104" t="n"/>
     </row>
     <row r="41" ht="50" customHeight="1">
       <c r="B41" s="85" t="inlineStr">
@@ -11916,81 +12281,82 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="75">
-    <mergeCell ref="C34:J34"/>
-    <mergeCell ref="B37:N37"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="M34:N34"/>
+  <mergeCells count="76">
+    <mergeCell ref="C33:J33"/>
+    <mergeCell ref="I3:N3"/>
+    <mergeCell ref="C35:J35"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="B37:M37"/>
+    <mergeCell ref="C25:J25"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I4:N4"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="C11:J11"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="C32:J32"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C33:J33"/>
     <mergeCell ref="C24:J24"/>
     <mergeCell ref="H41:I41"/>
+    <mergeCell ref="C26:J26"/>
+    <mergeCell ref="C10:J10"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="C9:J9"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="C36:J36"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="C28:J28"/>
+    <mergeCell ref="M34:N34"/>
     <mergeCell ref="M9:N9"/>
     <mergeCell ref="C14:J14"/>
-    <mergeCell ref="I3:N3"/>
     <mergeCell ref="B5:H5"/>
-    <mergeCell ref="C35:J35"/>
-    <mergeCell ref="C26:J26"/>
-    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="J41:N41"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C17:J17"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C34:J34"/>
+    <mergeCell ref="B42:G42"/>
     <mergeCell ref="C29:J29"/>
-    <mergeCell ref="M11:N11"/>
     <mergeCell ref="M20:N20"/>
-    <mergeCell ref="I5:N5"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="C25:J25"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="C10:J10"/>
-    <mergeCell ref="M31:N31"/>
     <mergeCell ref="C22:J22"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I4:N4"/>
     <mergeCell ref="C31:J31"/>
-    <mergeCell ref="B6:J6"/>
     <mergeCell ref="M22:N22"/>
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="C9:J9"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="M30:N30"/>
     <mergeCell ref="C12:J12"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="N37:Q37"/>
     <mergeCell ref="C21:J21"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="C11:J11"/>
     <mergeCell ref="M28:N28"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="C36:J36"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="J41:N41"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="M8:N8"/>
     <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="B16:J16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="C17:J17"/>
-    <mergeCell ref="M24:N24"/>
     <mergeCell ref="C7:J7"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="M23:N23"/>
     <mergeCell ref="M32:N32"/>
-    <mergeCell ref="C32:J32"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="C28:J28"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C19:J19"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Calender K1 Easy: corregir formato impresion (columnas y pagina igual que IMESA)
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -9872,6 +9872,22 @@
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
     <col width="12.77734375" customWidth="1" min="2" max="17"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.8" customHeight="1"/>
@@ -11062,42 +11078,46 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="9.5546875" customWidth="1" min="1" max="1"/>
+    <col width="12.77734375" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="7.8" customHeight="1">
       <c r="B1" s="83" t="inlineStr">
         <is>
           <t>AD-PACK  —  ÁREA DE CONVERSIÓN</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="56.55" customHeight="1">
       <c r="B2" s="84" t="inlineStr">
         <is>
           <t>MANTENIMIENTO PREVENTIVO   —   CALENDER K1 EASY</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3" ht="97.8" customHeight="1">
       <c r="B3" s="85" t="inlineStr">
         <is>
           <t>Alcance: Equipos de Conversión – AD-PACK</t>
@@ -11109,7 +11129,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4" ht="25.05" customHeight="1">
       <c r="B4" s="85" t="inlineStr">
         <is>
           <t>Tipo de mantenimiento:  Preventivo</t>
@@ -11121,7 +11141,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5" ht="46.2" customHeight="1">
       <c r="B5" s="85" t="inlineStr">
         <is>
           <t>Nombre de máquina:  Calender K1 Easy</t>
@@ -11133,7 +11153,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="25.05" customHeight="1">
       <c r="B6" s="86" t="inlineStr">
         <is>
           <t xml:space="preserve">  MECÁNICO</t>
@@ -11164,7 +11184,7 @@
       </c>
       <c r="N6" s="101" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="25.05" customHeight="1">
       <c r="B7" s="88" t="inlineStr">
         <is>
           <t>1</t>
@@ -11195,7 +11215,7 @@
       <c r="M7" s="91" t="n"/>
       <c r="N7" s="101" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="25.05" customHeight="1">
       <c r="B8" s="92" t="inlineStr">
         <is>
           <t>2</t>
@@ -11226,7 +11246,7 @@
       <c r="M8" s="95" t="n"/>
       <c r="N8" s="101" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="25.05" customHeight="1">
       <c r="B9" s="88" t="inlineStr">
         <is>
           <t>3</t>
@@ -11257,7 +11277,7 @@
       <c r="M9" s="91" t="n"/>
       <c r="N9" s="101" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="25.05" customHeight="1">
       <c r="B10" s="92" t="inlineStr">
         <is>
           <t>4</t>
@@ -11288,7 +11308,7 @@
       <c r="M10" s="95" t="n"/>
       <c r="N10" s="101" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="25.05" customHeight="1">
       <c r="B11" s="88" t="inlineStr">
         <is>
           <t>5</t>
@@ -11319,7 +11339,7 @@
       <c r="M11" s="91" t="n"/>
       <c r="N11" s="101" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="25.05" customHeight="1">
       <c r="B12" s="92" t="inlineStr">
         <is>
           <t>6</t>
@@ -11350,7 +11370,7 @@
       <c r="M12" s="95" t="n"/>
       <c r="N12" s="101" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="25.05" customHeight="1">
       <c r="B13" s="88" t="inlineStr">
         <is>
           <t>7</t>
@@ -11381,7 +11401,7 @@
       <c r="M13" s="91" t="n"/>
       <c r="N13" s="101" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="25.05" customHeight="1">
       <c r="B14" s="92" t="inlineStr">
         <is>
           <t>8</t>
@@ -11412,7 +11432,7 @@
       <c r="M14" s="95" t="n"/>
       <c r="N14" s="101" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="25.05" customHeight="1">
       <c r="B15" s="88" t="inlineStr">
         <is>
           <t>9</t>
@@ -11443,7 +11463,7 @@
       <c r="M15" s="91" t="n"/>
       <c r="N15" s="101" t="n"/>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16" ht="25.05" customHeight="1">
       <c r="B16" s="86" t="inlineStr">
         <is>
           <t xml:space="preserve">  ELÉCTRICO</t>
@@ -11474,7 +11494,7 @@
       </c>
       <c r="N16" s="101" t="n"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="25.05" customHeight="1">
       <c r="B17" s="88" t="inlineStr">
         <is>
           <t>10</t>
@@ -11505,7 +11525,7 @@
       <c r="M17" s="91" t="n"/>
       <c r="N17" s="101" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="25.05" customHeight="1">
       <c r="B18" s="92" t="inlineStr">
         <is>
           <t>11</t>
@@ -11536,7 +11556,7 @@
       <c r="M18" s="95" t="n"/>
       <c r="N18" s="101" t="n"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="25.05" customHeight="1">
       <c r="B19" s="88" t="inlineStr">
         <is>
           <t>12</t>
@@ -11567,7 +11587,7 @@
       <c r="M19" s="91" t="n"/>
       <c r="N19" s="101" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="25.05" customHeight="1">
       <c r="B20" s="92" t="inlineStr">
         <is>
           <t>13</t>
@@ -11598,7 +11618,7 @@
       <c r="M20" s="95" t="n"/>
       <c r="N20" s="101" t="n"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="25.05" customHeight="1">
       <c r="B21" s="88" t="inlineStr">
         <is>
           <t>14</t>
@@ -11629,7 +11649,7 @@
       <c r="M21" s="91" t="n"/>
       <c r="N21" s="101" t="n"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="25.05" customHeight="1">
       <c r="B22" s="92" t="inlineStr">
         <is>
           <t>15</t>
@@ -11660,7 +11680,7 @@
       <c r="M22" s="95" t="n"/>
       <c r="N22" s="101" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="25.05" customHeight="1">
       <c r="B23" s="88" t="inlineStr">
         <is>
           <t>16</t>
@@ -11691,7 +11711,7 @@
       <c r="M23" s="91" t="n"/>
       <c r="N23" s="101" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="25.05" customHeight="1">
       <c r="B24" s="92" t="inlineStr">
         <is>
           <t>17</t>
@@ -11722,7 +11742,7 @@
       <c r="M24" s="95" t="n"/>
       <c r="N24" s="101" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="25.05" customHeight="1">
       <c r="B25" s="88" t="inlineStr">
         <is>
           <t>18</t>
@@ -11753,7 +11773,7 @@
       <c r="M25" s="91" t="n"/>
       <c r="N25" s="101" t="n"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="25.05" customHeight="1">
       <c r="B26" s="92" t="inlineStr">
         <is>
           <t>19</t>
@@ -11784,7 +11804,7 @@
       <c r="M26" s="95" t="n"/>
       <c r="N26" s="101" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="25.05" customHeight="1">
       <c r="B27" s="88" t="inlineStr">
         <is>
           <t>20</t>
@@ -11815,7 +11835,7 @@
       <c r="M27" s="91" t="n"/>
       <c r="N27" s="101" t="n"/>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="25.05" customHeight="1">
       <c r="B28" s="92" t="inlineStr">
         <is>
           <t>21</t>
@@ -11846,7 +11866,7 @@
       <c r="M28" s="95" t="n"/>
       <c r="N28" s="101" t="n"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="25.05" customHeight="1">
       <c r="B29" s="88" t="inlineStr">
         <is>
           <t>22</t>
@@ -11877,7 +11897,7 @@
       <c r="M29" s="91" t="n"/>
       <c r="N29" s="101" t="n"/>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="25.05" customHeight="1">
       <c r="B30" s="86" t="inlineStr">
         <is>
           <t xml:space="preserve">  CALENTAMIENTO</t>
@@ -11908,7 +11928,7 @@
       </c>
       <c r="N30" s="101" t="n"/>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="25.05" customHeight="1">
       <c r="B31" s="88" t="inlineStr">
         <is>
           <t>23</t>
@@ -11939,7 +11959,7 @@
       <c r="M31" s="91" t="n"/>
       <c r="N31" s="101" t="n"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="25.05" customHeight="1">
       <c r="B32" s="92" t="inlineStr">
         <is>
           <t>24</t>
@@ -11970,7 +11990,7 @@
       <c r="M32" s="95" t="n"/>
       <c r="N32" s="101" t="n"/>
     </row>
-    <row r="33" ht="30" customHeight="1">
+    <row r="33" ht="25.05" customHeight="1">
       <c r="B33" s="88" t="inlineStr">
         <is>
           <t>25</t>
@@ -12282,84 +12302,85 @@
     </row>
   </sheetData>
   <mergeCells count="76">
+    <mergeCell ref="C34:J34"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="C15:J15"/>
     <mergeCell ref="C33:J33"/>
+    <mergeCell ref="C24:J24"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="C14:J14"/>
     <mergeCell ref="I3:N3"/>
+    <mergeCell ref="B5:H5"/>
     <mergeCell ref="C35:J35"/>
+    <mergeCell ref="C26:J26"/>
     <mergeCell ref="M35:N35"/>
+    <mergeCell ref="C29:J29"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="M20:N20"/>
     <mergeCell ref="I5:N5"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="B37:M37"/>
     <mergeCell ref="C25:J25"/>
     <mergeCell ref="M10:N10"/>
+    <mergeCell ref="C10:J10"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="C22:J22"/>
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="I4:N4"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="C31:J31"/>
     <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="C11:J11"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="B16:J16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="C32:J32"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C24:J24"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="C26:J26"/>
-    <mergeCell ref="C10:J10"/>
-    <mergeCell ref="B6:J6"/>
     <mergeCell ref="C9:J9"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="M7:N7"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="M22:N22"/>
     <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="C12:J12"/>
+    <mergeCell ref="N37:Q37"/>
+    <mergeCell ref="C21:J21"/>
+    <mergeCell ref="C11:J11"/>
+    <mergeCell ref="M6:N6"/>
     <mergeCell ref="B41:G41"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M36:N36"/>
     <mergeCell ref="C36:J36"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M33:N33"/>
     <mergeCell ref="M27:N27"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="C28:J28"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="C14:J14"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M12:N12"/>
     <mergeCell ref="C27:J27"/>
     <mergeCell ref="J41:N41"/>
     <mergeCell ref="B2:N2"/>
+    <mergeCell ref="M8:N8"/>
     <mergeCell ref="M26:N26"/>
+    <mergeCell ref="B16:J16"/>
     <mergeCell ref="C8:J8"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="C23:J23"/>
+    <mergeCell ref="M24:N24"/>
     <mergeCell ref="C17:J17"/>
+    <mergeCell ref="C7:J7"/>
     <mergeCell ref="M29:N29"/>
+    <mergeCell ref="B1:N1"/>
     <mergeCell ref="M23:N23"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="C32:J32"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="C28:J28"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C19:J19"/>
-    <mergeCell ref="C34:J34"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="C29:J29"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="C31:J31"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="C12:J12"/>
-    <mergeCell ref="N37:Q37"/>
-    <mergeCell ref="C21:J21"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="C23:J23"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M14:N14"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Calender K1 Easy: reconstruir hoja con estructura identica a Rotary Press (3 secciones, logos, formato correcto)
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -7217,7 +7217,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:Q39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
@@ -11078,1305 +11078,1535 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Q42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:Q42"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
-    <col width="12.77734375" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="12.77734375" customWidth="1" min="2" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="7.8" customHeight="1">
-      <c r="B1" s="83" t="inlineStr">
+    <row r="1" ht="7.8" customHeight="1"/>
+    <row r="2" ht="56.55" customHeight="1">
+      <c r="A2" s="11" t="n"/>
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>AD-PACK  —  ÁREA DE CONVERSIÓN</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="56.55" customHeight="1">
-      <c r="B2" s="84" t="inlineStr">
-        <is>
-          <t>MANTENIMIENTO PREVENTIVO   —   CALENDER K1 EASY</t>
-        </is>
-      </c>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="22" t="n"/>
+      <c r="F2" s="22" t="n"/>
+      <c r="G2" s="22" t="n"/>
+      <c r="H2" s="22" t="n"/>
+      <c r="I2" s="22" t="n"/>
+      <c r="J2" s="22" t="n"/>
+      <c r="K2" s="22" t="n"/>
+      <c r="L2" s="22" t="n"/>
+      <c r="M2" s="22" t="n"/>
+      <c r="N2" s="23" t="n"/>
+      <c r="O2" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> No. de Documento             A9.I1.F2
+ Revision:                                    00
+ Fecha:                        08/06/2026</t>
+        </is>
+      </c>
+      <c r="P2" s="50" t="n"/>
+      <c r="Q2" s="51" t="n"/>
     </row>
     <row r="3" ht="97.8" customHeight="1">
-      <c r="B3" s="85" t="inlineStr">
+      <c r="A3" s="11" t="n"/>
+      <c r="B3" s="36" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="38" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO PREVENTIVO   — Calender K1 Easy</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="n"/>
+      <c r="G3" s="22" t="n"/>
+      <c r="H3" s="22" t="n"/>
+      <c r="I3" s="22" t="n"/>
+      <c r="J3" s="22" t="n"/>
+      <c r="K3" s="22" t="n"/>
+      <c r="L3" s="22" t="n"/>
+      <c r="M3" s="22" t="n"/>
+      <c r="N3" s="23" t="n"/>
+      <c r="O3" s="35" t="n"/>
+      <c r="P3" s="22" t="n"/>
+      <c r="Q3" s="23" t="n"/>
+    </row>
+    <row r="4" ht="25.05" customHeight="1">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>Alcance: Equipos de Conversión – AD-PACK</t>
         </is>
       </c>
-      <c r="I3" s="85" t="inlineStr">
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="22" t="n"/>
+      <c r="H4" s="22" t="n"/>
+      <c r="I4" s="23" t="n"/>
+      <c r="J4" s="33" t="inlineStr">
         <is>
           <t>Autor: Mariano Leyva</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="25.05" customHeight="1">
-      <c r="B4" s="85" t="inlineStr">
+      <c r="K4" s="22" t="n"/>
+      <c r="L4" s="22" t="n"/>
+      <c r="M4" s="22" t="n"/>
+      <c r="N4" s="22" t="n"/>
+      <c r="O4" s="22" t="n"/>
+      <c r="P4" s="22" t="n"/>
+      <c r="Q4" s="23" t="n"/>
+    </row>
+    <row r="5" ht="46.2" customHeight="1">
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="37" t="inlineStr">
         <is>
           <t>Tipo de mantenimiento:  Preventivo</t>
         </is>
       </c>
-      <c r="I4" s="85" t="inlineStr">
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="22" t="n"/>
+      <c r="H5" s="22" t="n"/>
+      <c r="I5" s="23" t="n"/>
+      <c r="J5" s="33" t="inlineStr">
         <is>
           <t>Indicaciones: Usar EPP. Para revisiones eléctricas: PARO TOTAL.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="46.2" customHeight="1">
-      <c r="B5" s="85" t="inlineStr">
+      <c r="K5" s="22" t="n"/>
+      <c r="L5" s="22" t="n"/>
+      <c r="M5" s="22" t="n"/>
+      <c r="N5" s="22" t="n"/>
+      <c r="O5" s="22" t="n"/>
+      <c r="P5" s="22" t="n"/>
+      <c r="Q5" s="23" t="n"/>
+    </row>
+    <row r="6" ht="25.05" customHeight="1">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>Nombre de máquina:  Calender K1 Easy</t>
         </is>
       </c>
-      <c r="I5" s="85" t="inlineStr">
-        <is>
-          <t>Número de máquina:  K1-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="25.05" customHeight="1">
-      <c r="B6" s="86" t="inlineStr">
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="22" t="n"/>
+      <c r="H6" s="22" t="n"/>
+      <c r="I6" s="23" t="n"/>
+      <c r="J6" s="33" t="inlineStr">
+        <is>
+          <t>Número de máquina:  CK01</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="n"/>
+      <c r="L6" s="22" t="n"/>
+      <c r="M6" s="22" t="n"/>
+      <c r="N6" s="22" t="n"/>
+      <c r="O6" s="22" t="n"/>
+      <c r="P6" s="22" t="n"/>
+      <c r="Q6" s="23" t="n"/>
+    </row>
+    <row r="7" ht="25.05" customHeight="1">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  MECÁNICO</t>
         </is>
       </c>
-      <c r="C6" s="100" t="n"/>
-      <c r="D6" s="100" t="n"/>
-      <c r="E6" s="100" t="n"/>
-      <c r="F6" s="100" t="n"/>
-      <c r="G6" s="100" t="n"/>
-      <c r="H6" s="100" t="n"/>
-      <c r="I6" s="100" t="n"/>
-      <c r="J6" s="101" t="n"/>
-      <c r="K6" s="87" t="inlineStr">
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="22" t="n"/>
+      <c r="H7" s="22" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="23" t="n"/>
+      <c r="K7" s="1" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L6" s="87" t="inlineStr">
+      <c r="L7" s="27" t="inlineStr">
         <is>
           <t>NG</t>
         </is>
       </c>
-      <c r="M6" s="87" t="inlineStr">
+      <c r="M7" s="27" t="inlineStr">
         <is>
           <t>COMENTARIOS</t>
         </is>
       </c>
-      <c r="N6" s="101" t="n"/>
-    </row>
-    <row r="7" ht="25.05" customHeight="1">
-      <c r="B7" s="88" t="inlineStr">
+      <c r="N7" s="22" t="n"/>
+      <c r="O7" s="22" t="n"/>
+      <c r="P7" s="22" t="n"/>
+      <c r="Q7" s="23" t="n"/>
+    </row>
+    <row r="8" ht="25.05" customHeight="1">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C7" s="89" t="inlineStr">
+      <c r="C8" s="26" t="inlineStr">
         <is>
           <t>Inspección visual: ruidos, vibraciones y fugas en rodillos</t>
         </is>
       </c>
-      <c r="D7" s="100" t="n"/>
-      <c r="E7" s="100" t="n"/>
-      <c r="F7" s="100" t="n"/>
-      <c r="G7" s="100" t="n"/>
-      <c r="H7" s="100" t="n"/>
-      <c r="I7" s="100" t="n"/>
-      <c r="J7" s="101" t="n"/>
-      <c r="K7" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L7" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M7" s="91" t="n"/>
-      <c r="N7" s="101" t="n"/>
-    </row>
-    <row r="8" ht="25.05" customHeight="1">
-      <c r="B8" s="92" t="inlineStr">
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="22" t="n"/>
+      <c r="H8" s="22" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="23" t="n"/>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M8" s="21" t="n"/>
+      <c r="N8" s="22" t="n"/>
+      <c r="O8" s="22" t="n"/>
+      <c r="P8" s="22" t="n"/>
+      <c r="Q8" s="23" t="n"/>
+    </row>
+    <row r="9" ht="25.05" customHeight="1">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C8" s="93" t="inlineStr">
+      <c r="C9" s="26" t="inlineStr">
         <is>
           <t>Lubricación de rodillos de calandria (baleros y chumaceras)</t>
         </is>
       </c>
-      <c r="D8" s="100" t="n"/>
-      <c r="E8" s="100" t="n"/>
-      <c r="F8" s="100" t="n"/>
-      <c r="G8" s="100" t="n"/>
-      <c r="H8" s="100" t="n"/>
-      <c r="I8" s="100" t="n"/>
-      <c r="J8" s="101" t="n"/>
-      <c r="K8" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L8" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M8" s="95" t="n"/>
-      <c r="N8" s="101" t="n"/>
-    </row>
-    <row r="9" ht="25.05" customHeight="1">
-      <c r="B9" s="88" t="inlineStr">
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="22" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="23" t="n"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M9" s="21" t="n"/>
+      <c r="N9" s="22" t="n"/>
+      <c r="O9" s="22" t="n"/>
+      <c r="P9" s="22" t="n"/>
+      <c r="Q9" s="23" t="n"/>
+    </row>
+    <row r="10" ht="25.05" customHeight="1">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C9" s="89" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
         <is>
           <t>Revisión y lubricación de cadena de transmisión y sprockets</t>
         </is>
       </c>
-      <c r="D9" s="100" t="n"/>
-      <c r="E9" s="100" t="n"/>
-      <c r="F9" s="100" t="n"/>
-      <c r="G9" s="100" t="n"/>
-      <c r="H9" s="100" t="n"/>
-      <c r="I9" s="100" t="n"/>
-      <c r="J9" s="101" t="n"/>
-      <c r="K9" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L9" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M9" s="91" t="n"/>
-      <c r="N9" s="101" t="n"/>
-    </row>
-    <row r="10" ht="25.05" customHeight="1">
-      <c r="B10" s="92" t="inlineStr">
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="22" t="n"/>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="23" t="n"/>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M10" s="21" t="n"/>
+      <c r="N10" s="22" t="n"/>
+      <c r="O10" s="22" t="n"/>
+      <c r="P10" s="22" t="n"/>
+      <c r="Q10" s="23" t="n"/>
+    </row>
+    <row r="11" ht="25.05" customHeight="1">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C10" s="93" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
         <is>
           <t>Verificación de tensión de cadena (deflexión máx. 1% de longitud)</t>
         </is>
       </c>
-      <c r="D10" s="100" t="n"/>
-      <c r="E10" s="100" t="n"/>
-      <c r="F10" s="100" t="n"/>
-      <c r="G10" s="100" t="n"/>
-      <c r="H10" s="100" t="n"/>
-      <c r="I10" s="100" t="n"/>
-      <c r="J10" s="101" t="n"/>
-      <c r="K10" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L10" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M10" s="95" t="n"/>
-      <c r="N10" s="101" t="n"/>
-    </row>
-    <row r="11" ht="25.05" customHeight="1">
-      <c r="B11" s="88" t="inlineStr">
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="22" t="n"/>
+      <c r="H11" s="22" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M11" s="21" t="n"/>
+      <c r="N11" s="22" t="n"/>
+      <c r="O11" s="22" t="n"/>
+      <c r="P11" s="22" t="n"/>
+      <c r="Q11" s="23" t="n"/>
+    </row>
+    <row r="12" ht="25.05" customHeight="1">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C11" s="89" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>Revisión de caja reductora: nivel y calidad de aceite</t>
         </is>
       </c>
-      <c r="D11" s="100" t="n"/>
-      <c r="E11" s="100" t="n"/>
-      <c r="F11" s="100" t="n"/>
-      <c r="G11" s="100" t="n"/>
-      <c r="H11" s="100" t="n"/>
-      <c r="I11" s="100" t="n"/>
-      <c r="J11" s="101" t="n"/>
-      <c r="K11" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L11" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M11" s="91" t="n"/>
-      <c r="N11" s="101" t="n"/>
-    </row>
-    <row r="12" ht="25.05" customHeight="1">
-      <c r="B12" s="92" t="inlineStr">
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
+      <c r="G12" s="22" t="n"/>
+      <c r="H12" s="22" t="n"/>
+      <c r="I12" s="22" t="n"/>
+      <c r="J12" s="23" t="n"/>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M12" s="21" t="n"/>
+      <c r="N12" s="22" t="n"/>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="22" t="n"/>
+      <c r="Q12" s="23" t="n"/>
+    </row>
+    <row r="13" ht="25.05" customHeight="1">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C12" s="93" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
         <is>
           <t>Verificación de alineación y paralelismo de rodillos</t>
         </is>
       </c>
-      <c r="D12" s="100" t="n"/>
-      <c r="E12" s="100" t="n"/>
-      <c r="F12" s="100" t="n"/>
-      <c r="G12" s="100" t="n"/>
-      <c r="H12" s="100" t="n"/>
-      <c r="I12" s="100" t="n"/>
-      <c r="J12" s="101" t="n"/>
-      <c r="K12" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L12" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M12" s="95" t="n"/>
-      <c r="N12" s="101" t="n"/>
-    </row>
-    <row r="13" ht="25.05" customHeight="1">
-      <c r="B13" s="88" t="inlineStr">
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="22" t="n"/>
+      <c r="G13" s="22" t="n"/>
+      <c r="H13" s="22" t="n"/>
+      <c r="I13" s="22" t="n"/>
+      <c r="J13" s="23" t="n"/>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M13" s="21" t="n"/>
+      <c r="N13" s="22" t="n"/>
+      <c r="O13" s="22" t="n"/>
+      <c r="P13" s="22" t="n"/>
+      <c r="Q13" s="23" t="n"/>
+    </row>
+    <row r="14" ht="25.05" customHeight="1">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C13" s="89" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>Limpieza de rodillos y superficie de contacto (residuos de material)</t>
         </is>
       </c>
-      <c r="D13" s="100" t="n"/>
-      <c r="E13" s="100" t="n"/>
-      <c r="F13" s="100" t="n"/>
-      <c r="G13" s="100" t="n"/>
-      <c r="H13" s="100" t="n"/>
-      <c r="I13" s="100" t="n"/>
-      <c r="J13" s="101" t="n"/>
-      <c r="K13" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L13" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M13" s="91" t="n"/>
-      <c r="N13" s="101" t="n"/>
-    </row>
-    <row r="14" ht="25.05" customHeight="1">
-      <c r="B14" s="92" t="inlineStr">
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="22" t="n"/>
+      <c r="G14" s="22" t="n"/>
+      <c r="H14" s="22" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="23" t="n"/>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M14" s="21" t="n"/>
+      <c r="N14" s="22" t="n"/>
+      <c r="O14" s="22" t="n"/>
+      <c r="P14" s="22" t="n"/>
+      <c r="Q14" s="23" t="n"/>
+    </row>
+    <row r="15" ht="25.05" customHeight="1">
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C14" s="93" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
         <is>
           <t>Revisión de tornillería y fijaciones estructurales</t>
         </is>
       </c>
-      <c r="D14" s="100" t="n"/>
-      <c r="E14" s="100" t="n"/>
-      <c r="F14" s="100" t="n"/>
-      <c r="G14" s="100" t="n"/>
-      <c r="H14" s="100" t="n"/>
-      <c r="I14" s="100" t="n"/>
-      <c r="J14" s="101" t="n"/>
-      <c r="K14" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L14" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M14" s="95" t="n"/>
-      <c r="N14" s="101" t="n"/>
-    </row>
-    <row r="15" ht="25.05" customHeight="1">
-      <c r="B15" s="88" t="inlineStr">
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="22" t="n"/>
+      <c r="G15" s="22" t="n"/>
+      <c r="H15" s="22" t="n"/>
+      <c r="I15" s="22" t="n"/>
+      <c r="J15" s="23" t="n"/>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M15" s="21" t="n"/>
+      <c r="N15" s="22" t="n"/>
+      <c r="O15" s="22" t="n"/>
+      <c r="P15" s="22" t="n"/>
+      <c r="Q15" s="23" t="n"/>
+    </row>
+    <row r="16" ht="25.05" customHeight="1">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C15" s="89" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Verificación del servo motor TECO JSMA-PSC44BK (temperatura y vibración)</t>
         </is>
       </c>
-      <c r="D15" s="100" t="n"/>
-      <c r="E15" s="100" t="n"/>
-      <c r="F15" s="100" t="n"/>
-      <c r="G15" s="100" t="n"/>
-      <c r="H15" s="100" t="n"/>
-      <c r="I15" s="100" t="n"/>
-      <c r="J15" s="101" t="n"/>
-      <c r="K15" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L15" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M15" s="91" t="n"/>
-      <c r="N15" s="101" t="n"/>
-    </row>
-    <row r="16" ht="25.05" customHeight="1">
-      <c r="B16" s="86" t="inlineStr">
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="22" t="n"/>
+      <c r="G16" s="22" t="n"/>
+      <c r="H16" s="22" t="n"/>
+      <c r="I16" s="22" t="n"/>
+      <c r="J16" s="23" t="n"/>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M16" s="21" t="n"/>
+      <c r="N16" s="22" t="n"/>
+      <c r="O16" s="22" t="n"/>
+      <c r="P16" s="22" t="n"/>
+      <c r="Q16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="25.05" customHeight="1">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  ELÉCTRICO</t>
         </is>
       </c>
-      <c r="C16" s="100" t="n"/>
-      <c r="D16" s="100" t="n"/>
-      <c r="E16" s="100" t="n"/>
-      <c r="F16" s="100" t="n"/>
-      <c r="G16" s="100" t="n"/>
-      <c r="H16" s="100" t="n"/>
-      <c r="I16" s="100" t="n"/>
-      <c r="J16" s="101" t="n"/>
-      <c r="K16" s="87" t="inlineStr">
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="22" t="n"/>
+      <c r="G17" s="22" t="n"/>
+      <c r="H17" s="22" t="n"/>
+      <c r="I17" s="22" t="n"/>
+      <c r="J17" s="23" t="n"/>
+      <c r="K17" s="1" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L16" s="87" t="inlineStr">
+      <c r="L17" s="27" t="inlineStr">
         <is>
           <t>NG</t>
         </is>
       </c>
-      <c r="M16" s="87" t="inlineStr">
+      <c r="M17" s="27" t="inlineStr">
         <is>
           <t>COMENTARIOS</t>
         </is>
       </c>
-      <c r="N16" s="101" t="n"/>
-    </row>
-    <row r="17" ht="25.05" customHeight="1">
-      <c r="B17" s="88" t="inlineStr">
+      <c r="N17" s="22" t="n"/>
+      <c r="O17" s="22" t="n"/>
+      <c r="P17" s="22" t="n"/>
+      <c r="Q17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="25.05" customHeight="1">
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C17" s="89" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>Verificación del HMI MCU 01 TS: alarmas, indicadores y pantalla táctil</t>
         </is>
       </c>
-      <c r="D17" s="100" t="n"/>
-      <c r="E17" s="100" t="n"/>
-      <c r="F17" s="100" t="n"/>
-      <c r="G17" s="100" t="n"/>
-      <c r="H17" s="100" t="n"/>
-      <c r="I17" s="100" t="n"/>
-      <c r="J17" s="101" t="n"/>
-      <c r="K17" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L17" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M17" s="91" t="n"/>
-      <c r="N17" s="101" t="n"/>
-    </row>
-    <row r="18" ht="25.05" customHeight="1">
-      <c r="B18" s="92" t="inlineStr">
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="22" t="n"/>
+      <c r="G18" s="22" t="n"/>
+      <c r="H18" s="22" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="23" t="n"/>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M18" s="21" t="n"/>
+      <c r="N18" s="22" t="n"/>
+      <c r="O18" s="22" t="n"/>
+      <c r="P18" s="22" t="n"/>
+      <c r="Q18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="25.05" customHeight="1">
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="C18" s="93" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>Limpieza de tablero eléctrico y revisión de cableado y ducterías</t>
         </is>
       </c>
-      <c r="D18" s="100" t="n"/>
-      <c r="E18" s="100" t="n"/>
-      <c r="F18" s="100" t="n"/>
-      <c r="G18" s="100" t="n"/>
-      <c r="H18" s="100" t="n"/>
-      <c r="I18" s="100" t="n"/>
-      <c r="J18" s="101" t="n"/>
-      <c r="K18" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L18" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M18" s="95" t="n"/>
-      <c r="N18" s="101" t="n"/>
-    </row>
-    <row r="19" ht="25.05" customHeight="1">
-      <c r="B19" s="88" t="inlineStr">
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="22" t="n"/>
+      <c r="F19" s="22" t="n"/>
+      <c r="G19" s="22" t="n"/>
+      <c r="H19" s="22" t="n"/>
+      <c r="I19" s="22" t="n"/>
+      <c r="J19" s="23" t="n"/>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M19" s="21" t="n"/>
+      <c r="N19" s="22" t="n"/>
+      <c r="O19" s="22" t="n"/>
+      <c r="P19" s="22" t="n"/>
+      <c r="Q19" s="23" t="n"/>
+    </row>
+    <row r="20" ht="25.05" customHeight="1">
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C19" s="89" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>Reapriete de terminales y conexiones eléctricas</t>
         </is>
       </c>
-      <c r="D19" s="100" t="n"/>
-      <c r="E19" s="100" t="n"/>
-      <c r="F19" s="100" t="n"/>
-      <c r="G19" s="100" t="n"/>
-      <c r="H19" s="100" t="n"/>
-      <c r="I19" s="100" t="n"/>
-      <c r="J19" s="101" t="n"/>
-      <c r="K19" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L19" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M19" s="91" t="n"/>
-      <c r="N19" s="101" t="n"/>
-    </row>
-    <row r="20" ht="25.05" customHeight="1">
-      <c r="B20" s="92" t="inlineStr">
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="22" t="n"/>
+      <c r="G20" s="22" t="n"/>
+      <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="23" t="n"/>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M20" s="21" t="n"/>
+      <c r="N20" s="22" t="n"/>
+      <c r="O20" s="22" t="n"/>
+      <c r="P20" s="22" t="n"/>
+      <c r="Q20" s="23" t="n"/>
+    </row>
+    <row r="21" ht="25.05" customHeight="1">
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="C20" s="93" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
         <is>
           <t>Revisión de portafusibles Lovato FB01 B 2P: 2FU1, 6FU1, 7FU1</t>
         </is>
       </c>
-      <c r="D20" s="100" t="n"/>
-      <c r="E20" s="100" t="n"/>
-      <c r="F20" s="100" t="n"/>
-      <c r="G20" s="100" t="n"/>
-      <c r="H20" s="100" t="n"/>
-      <c r="I20" s="100" t="n"/>
-      <c r="J20" s="101" t="n"/>
-      <c r="K20" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L20" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M20" s="95" t="n"/>
-      <c r="N20" s="101" t="n"/>
-    </row>
-    <row r="21" ht="25.05" customHeight="1">
-      <c r="B21" s="88" t="inlineStr">
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="22" t="n"/>
+      <c r="F21" s="22" t="n"/>
+      <c r="G21" s="22" t="n"/>
+      <c r="H21" s="22" t="n"/>
+      <c r="I21" s="22" t="n"/>
+      <c r="J21" s="23" t="n"/>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M21" s="27" t="n"/>
+      <c r="N21" s="22" t="n"/>
+      <c r="O21" s="22" t="n"/>
+      <c r="P21" s="22" t="n"/>
+      <c r="Q21" s="23" t="n"/>
+    </row>
+    <row r="22" ht="25.05" customHeight="1">
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C21" s="89" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>Verificación del relé de seguridad Allen-Bradley MSR126.1T (7K1)</t>
         </is>
       </c>
-      <c r="D21" s="100" t="n"/>
-      <c r="E21" s="100" t="n"/>
-      <c r="F21" s="100" t="n"/>
-      <c r="G21" s="100" t="n"/>
-      <c r="H21" s="100" t="n"/>
-      <c r="I21" s="100" t="n"/>
-      <c r="J21" s="101" t="n"/>
-      <c r="K21" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L21" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M21" s="91" t="n"/>
-      <c r="N21" s="101" t="n"/>
-    </row>
-    <row r="22" ht="25.05" customHeight="1">
-      <c r="B22" s="92" t="inlineStr">
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="22" t="n"/>
+      <c r="F22" s="22" t="n"/>
+      <c r="G22" s="22" t="n"/>
+      <c r="H22" s="22" t="n"/>
+      <c r="I22" s="22" t="n"/>
+      <c r="J22" s="23" t="n"/>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M22" s="21" t="n"/>
+      <c r="N22" s="22" t="n"/>
+      <c r="O22" s="22" t="n"/>
+      <c r="P22" s="22" t="n"/>
+      <c r="Q22" s="23" t="n"/>
+    </row>
+    <row r="23" ht="25.05" customHeight="1">
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C22" s="93" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>Revisión del servo drive TECO: parámetros, fallas y conexiones</t>
         </is>
       </c>
-      <c r="D22" s="100" t="n"/>
-      <c r="E22" s="100" t="n"/>
-      <c r="F22" s="100" t="n"/>
-      <c r="G22" s="100" t="n"/>
-      <c r="H22" s="100" t="n"/>
-      <c r="I22" s="100" t="n"/>
-      <c r="J22" s="101" t="n"/>
-      <c r="K22" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L22" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M22" s="95" t="n"/>
-      <c r="N22" s="101" t="n"/>
-    </row>
-    <row r="23" ht="25.05" customHeight="1">
-      <c r="B23" s="88" t="inlineStr">
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="22" t="n"/>
+      <c r="F23" s="22" t="n"/>
+      <c r="G23" s="22" t="n"/>
+      <c r="H23" s="22" t="n"/>
+      <c r="I23" s="22" t="n"/>
+      <c r="J23" s="23" t="n"/>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M23" s="21" t="n"/>
+      <c r="N23" s="22" t="n"/>
+      <c r="O23" s="22" t="n"/>
+      <c r="P23" s="22" t="n"/>
+      <c r="Q23" s="23" t="n"/>
+    </row>
+    <row r="24" ht="25.05" customHeight="1">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C23" s="89" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
         <is>
           <t>Verificación de fuente de poder Omron S8VK-C12024 (salida 24 VDC)</t>
         </is>
       </c>
-      <c r="D23" s="100" t="n"/>
-      <c r="E23" s="100" t="n"/>
-      <c r="F23" s="100" t="n"/>
-      <c r="G23" s="100" t="n"/>
-      <c r="H23" s="100" t="n"/>
-      <c r="I23" s="100" t="n"/>
-      <c r="J23" s="101" t="n"/>
-      <c r="K23" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L23" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M23" s="91" t="n"/>
-      <c r="N23" s="101" t="n"/>
-    </row>
-    <row r="24" ht="25.05" customHeight="1">
-      <c r="B24" s="92" t="inlineStr">
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="22" t="n"/>
+      <c r="G24" s="22" t="n"/>
+      <c r="H24" s="22" t="n"/>
+      <c r="I24" s="22" t="n"/>
+      <c r="J24" s="23" t="n"/>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M24" s="21" t="n"/>
+      <c r="N24" s="22" t="n"/>
+      <c r="O24" s="22" t="n"/>
+      <c r="P24" s="22" t="n"/>
+      <c r="Q24" s="23" t="n"/>
+    </row>
+    <row r="25" ht="25.05" customHeight="1">
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C24" s="93" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>Revisión del relevador SSR RM1A48D50 (7KPR1): temperatura y sujeción</t>
         </is>
       </c>
-      <c r="D24" s="100" t="n"/>
-      <c r="E24" s="100" t="n"/>
-      <c r="F24" s="100" t="n"/>
-      <c r="G24" s="100" t="n"/>
-      <c r="H24" s="100" t="n"/>
-      <c r="I24" s="100" t="n"/>
-      <c r="J24" s="101" t="n"/>
-      <c r="K24" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L24" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M24" s="95" t="n"/>
-      <c r="N24" s="101" t="n"/>
-    </row>
-    <row r="25" ht="25.05" customHeight="1">
-      <c r="B25" s="88" t="inlineStr">
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="22" t="n"/>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="22" t="n"/>
+      <c r="J25" s="23" t="n"/>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M25" s="21" t="n"/>
+      <c r="N25" s="22" t="n"/>
+      <c r="O25" s="22" t="n"/>
+      <c r="P25" s="22" t="n"/>
+      <c r="Q25" s="23" t="n"/>
+    </row>
+    <row r="26" ht="25.05" customHeight="1">
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="C25" s="89" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>Prueba funcional: paro de emergencia y botón REAJUSTE EMERGENCIA</t>
         </is>
       </c>
-      <c r="D25" s="100" t="n"/>
-      <c r="E25" s="100" t="n"/>
-      <c r="F25" s="100" t="n"/>
-      <c r="G25" s="100" t="n"/>
-      <c r="H25" s="100" t="n"/>
-      <c r="I25" s="100" t="n"/>
-      <c r="J25" s="101" t="n"/>
-      <c r="K25" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L25" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M25" s="91" t="n"/>
-      <c r="N25" s="101" t="n"/>
-    </row>
-    <row r="26" ht="25.05" customHeight="1">
-      <c r="B26" s="92" t="inlineStr">
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="22" t="n"/>
+      <c r="F26" s="22" t="n"/>
+      <c r="G26" s="22" t="n"/>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="22" t="n"/>
+      <c r="J26" s="23" t="n"/>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M26" s="21" t="n"/>
+      <c r="N26" s="22" t="n"/>
+      <c r="O26" s="22" t="n"/>
+      <c r="P26" s="22" t="n"/>
+      <c r="Q26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="25.05" customHeight="1">
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="C26" s="93" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>Verificación de interruptor de seguridad Pizzato (funcionamiento y ajuste)</t>
         </is>
       </c>
-      <c r="D26" s="100" t="n"/>
-      <c r="E26" s="100" t="n"/>
-      <c r="F26" s="100" t="n"/>
-      <c r="G26" s="100" t="n"/>
-      <c r="H26" s="100" t="n"/>
-      <c r="I26" s="100" t="n"/>
-      <c r="J26" s="101" t="n"/>
-      <c r="K26" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L26" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M26" s="95" t="n"/>
-      <c r="N26" s="101" t="n"/>
-    </row>
-    <row r="27" ht="25.05" customHeight="1">
-      <c r="B27" s="88" t="inlineStr">
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="22" t="n"/>
+      <c r="G27" s="22" t="n"/>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="22" t="n"/>
+      <c r="J27" s="23" t="n"/>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M27" s="63" t="n"/>
+      <c r="N27" s="81" t="n"/>
+      <c r="O27" s="81" t="n"/>
+      <c r="P27" s="81" t="n"/>
+      <c r="Q27" s="82" t="n"/>
+    </row>
+    <row r="28" ht="25.05" customHeight="1">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C27" s="89" t="inlineStr">
+      <c r="C28" s="26" t="inlineStr">
         <is>
           <t>Revisión del módulo I/O SHS DIN (señales de entrada/salida)</t>
         </is>
       </c>
-      <c r="D27" s="100" t="n"/>
-      <c r="E27" s="100" t="n"/>
-      <c r="F27" s="100" t="n"/>
-      <c r="G27" s="100" t="n"/>
-      <c r="H27" s="100" t="n"/>
-      <c r="I27" s="100" t="n"/>
-      <c r="J27" s="101" t="n"/>
-      <c r="K27" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L27" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M27" s="91" t="n"/>
-      <c r="N27" s="101" t="n"/>
-    </row>
-    <row r="28" ht="25.05" customHeight="1">
-      <c r="B28" s="92" t="inlineStr">
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="22" t="n"/>
+      <c r="G28" s="22" t="n"/>
+      <c r="H28" s="22" t="n"/>
+      <c r="I28" s="22" t="n"/>
+      <c r="J28" s="23" t="n"/>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M28" s="66" t="n"/>
+      <c r="N28" s="50" t="n"/>
+      <c r="O28" s="50" t="n"/>
+      <c r="P28" s="50" t="n"/>
+      <c r="Q28" s="51" t="n"/>
+    </row>
+    <row r="29" ht="25.05" customHeight="1">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="C28" s="93" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
         <is>
           <t>Verificación del interruptor principal ABB OT25F4N2 (2QS1)</t>
         </is>
       </c>
-      <c r="D28" s="100" t="n"/>
-      <c r="E28" s="100" t="n"/>
-      <c r="F28" s="100" t="n"/>
-      <c r="G28" s="100" t="n"/>
-      <c r="H28" s="100" t="n"/>
-      <c r="I28" s="100" t="n"/>
-      <c r="J28" s="101" t="n"/>
-      <c r="K28" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L28" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M28" s="95" t="n"/>
-      <c r="N28" s="101" t="n"/>
-    </row>
-    <row r="29" ht="25.05" customHeight="1">
-      <c r="B29" s="88" t="inlineStr">
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="22" t="n"/>
+      <c r="G29" s="22" t="n"/>
+      <c r="H29" s="22" t="n"/>
+      <c r="I29" s="22" t="n"/>
+      <c r="J29" s="23" t="n"/>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M29" s="66" t="n"/>
+      <c r="N29" s="50" t="n"/>
+      <c r="O29" s="50" t="n"/>
+      <c r="P29" s="50" t="n"/>
+      <c r="Q29" s="51" t="n"/>
+    </row>
+    <row r="30" ht="25.05" customHeight="1">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="C29" s="89" t="inlineStr">
+      <c r="C30" s="26" t="inlineStr">
         <is>
           <t>Verificación de tierras físicas y continuidad de tierra</t>
         </is>
       </c>
-      <c r="D29" s="100" t="n"/>
-      <c r="E29" s="100" t="n"/>
-      <c r="F29" s="100" t="n"/>
-      <c r="G29" s="100" t="n"/>
-      <c r="H29" s="100" t="n"/>
-      <c r="I29" s="100" t="n"/>
-      <c r="J29" s="101" t="n"/>
-      <c r="K29" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L29" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M29" s="91" t="n"/>
-      <c r="N29" s="101" t="n"/>
-    </row>
-    <row r="30" ht="25.05" customHeight="1">
-      <c r="B30" s="86" t="inlineStr">
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="22" t="n"/>
+      <c r="F30" s="22" t="n"/>
+      <c r="G30" s="22" t="n"/>
+      <c r="H30" s="22" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M30" s="66" t="n"/>
+      <c r="N30" s="50" t="n"/>
+      <c r="O30" s="50" t="n"/>
+      <c r="P30" s="50" t="n"/>
+      <c r="Q30" s="51" t="n"/>
+    </row>
+    <row r="31" ht="25.05" customHeight="1">
+      <c r="B31" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  CALENTAMIENTO</t>
         </is>
       </c>
-      <c r="C30" s="100" t="n"/>
-      <c r="D30" s="100" t="n"/>
-      <c r="E30" s="100" t="n"/>
-      <c r="F30" s="100" t="n"/>
-      <c r="G30" s="100" t="n"/>
-      <c r="H30" s="100" t="n"/>
-      <c r="I30" s="100" t="n"/>
-      <c r="J30" s="101" t="n"/>
-      <c r="K30" s="87" t="inlineStr">
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="22" t="n"/>
+      <c r="G31" s="22" t="n"/>
+      <c r="H31" s="22" t="n"/>
+      <c r="I31" s="22" t="n"/>
+      <c r="J31" s="23" t="n"/>
+      <c r="K31" s="1" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="L30" s="87" t="inlineStr">
+      <c r="L31" s="27" t="inlineStr">
         <is>
           <t>NG</t>
         </is>
       </c>
-      <c r="M30" s="87" t="inlineStr">
+      <c r="M31" s="27" t="inlineStr">
         <is>
           <t>COMENTARIOS</t>
         </is>
       </c>
-      <c r="N30" s="101" t="n"/>
-    </row>
-    <row r="31" ht="25.05" customHeight="1">
-      <c r="B31" s="88" t="inlineStr">
+      <c r="N31" s="22" t="n"/>
+      <c r="O31" s="22" t="n"/>
+      <c r="P31" s="22" t="n"/>
+      <c r="Q31" s="23" t="n"/>
+    </row>
+    <row r="32" ht="25.05" customHeight="1">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="C31" s="89" t="inlineStr">
+      <c r="C32" s="26" t="inlineStr">
         <is>
           <t>Verificación de temperatura de trabajo de rodillos calefactores</t>
         </is>
       </c>
-      <c r="D31" s="100" t="n"/>
-      <c r="E31" s="100" t="n"/>
-      <c r="F31" s="100" t="n"/>
-      <c r="G31" s="100" t="n"/>
-      <c r="H31" s="100" t="n"/>
-      <c r="I31" s="100" t="n"/>
-      <c r="J31" s="101" t="n"/>
-      <c r="K31" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L31" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M31" s="91" t="n"/>
-      <c r="N31" s="101" t="n"/>
-    </row>
-    <row r="32" ht="25.05" customHeight="1">
-      <c r="B32" s="92" t="inlineStr">
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="22" t="n"/>
+      <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M32" s="66" t="n"/>
+      <c r="N32" s="50" t="n"/>
+      <c r="O32" s="50" t="n"/>
+      <c r="P32" s="50" t="n"/>
+      <c r="Q32" s="51" t="n"/>
+    </row>
+    <row r="33" ht="25.05" customHeight="1">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="C32" s="93" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
         <is>
           <t>Limpieza de resistencias calefactoras (polvo y residuos de material)</t>
         </is>
       </c>
-      <c r="D32" s="100" t="n"/>
-      <c r="E32" s="100" t="n"/>
-      <c r="F32" s="100" t="n"/>
-      <c r="G32" s="100" t="n"/>
-      <c r="H32" s="100" t="n"/>
-      <c r="I32" s="100" t="n"/>
-      <c r="J32" s="101" t="n"/>
-      <c r="K32" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L32" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M32" s="95" t="n"/>
-      <c r="N32" s="101" t="n"/>
-    </row>
-    <row r="33" ht="25.05" customHeight="1">
-      <c r="B33" s="88" t="inlineStr">
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="22" t="n"/>
+      <c r="F33" s="22" t="n"/>
+      <c r="G33" s="22" t="n"/>
+      <c r="H33" s="22" t="n"/>
+      <c r="I33" s="22" t="n"/>
+      <c r="J33" s="23" t="n"/>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M33" s="66" t="n"/>
+      <c r="N33" s="50" t="n"/>
+      <c r="O33" s="50" t="n"/>
+      <c r="P33" s="50" t="n"/>
+      <c r="Q33" s="51" t="n"/>
+    </row>
+    <row r="34" ht="17.4" customHeight="1">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="C33" s="89" t="inlineStr">
+      <c r="C34" s="26" t="inlineStr">
         <is>
           <t>Calibración de termocuplas y verificación de control de temperatura</t>
         </is>
       </c>
-      <c r="D33" s="100" t="n"/>
-      <c r="E33" s="100" t="n"/>
-      <c r="F33" s="100" t="n"/>
-      <c r="G33" s="100" t="n"/>
-      <c r="H33" s="100" t="n"/>
-      <c r="I33" s="100" t="n"/>
-      <c r="J33" s="101" t="n"/>
-      <c r="K33" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L33" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M33" s="91" t="n"/>
-      <c r="N33" s="101" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="B34" s="92" t="inlineStr">
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="22" t="n"/>
+      <c r="G34" s="22" t="n"/>
+      <c r="H34" s="22" t="n"/>
+      <c r="I34" s="22" t="n"/>
+      <c r="J34" s="23" t="n"/>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M34" s="23" t="n"/>
+      <c r="N34" s="22" t="n"/>
+      <c r="O34" s="22" t="n"/>
+      <c r="P34" s="22" t="n"/>
+      <c r="Q34" s="23" t="n"/>
+    </row>
+    <row r="35" ht="17.4" customHeight="1">
+      <c r="A35" s="11" t="n"/>
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="C34" s="93" t="inlineStr">
+      <c r="C35" s="26" t="inlineStr">
         <is>
           <t>Medición eléctrica de resistencias calefactoras: continuidad y ohms</t>
         </is>
       </c>
-      <c r="D34" s="100" t="n"/>
-      <c r="E34" s="100" t="n"/>
-      <c r="F34" s="100" t="n"/>
-      <c r="G34" s="100" t="n"/>
-      <c r="H34" s="100" t="n"/>
-      <c r="I34" s="100" t="n"/>
-      <c r="J34" s="101" t="n"/>
-      <c r="K34" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L34" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M34" s="95" t="n"/>
-      <c r="N34" s="101" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="88" t="inlineStr">
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="22" t="n"/>
+      <c r="G35" s="22" t="n"/>
+      <c r="H35" s="22" t="n"/>
+      <c r="I35" s="22" t="n"/>
+      <c r="J35" s="23" t="n"/>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="n"/>
+      <c r="N35" s="22" t="n"/>
+      <c r="O35" s="22" t="n"/>
+      <c r="P35" s="22" t="n"/>
+      <c r="Q35" s="23" t="n"/>
+    </row>
+    <row r="36" ht="17.4" customHeight="1">
+      <c r="A36" s="11" t="n"/>
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="C35" s="89" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>Verificación del SSR RM1A48D50 como control de calefacción (7KPR1)</t>
         </is>
       </c>
-      <c r="D35" s="100" t="n"/>
-      <c r="E35" s="100" t="n"/>
-      <c r="F35" s="100" t="n"/>
-      <c r="G35" s="100" t="n"/>
-      <c r="H35" s="100" t="n"/>
-      <c r="I35" s="100" t="n"/>
-      <c r="J35" s="101" t="n"/>
-      <c r="K35" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L35" s="90" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M35" s="91" t="n"/>
-      <c r="N35" s="101" t="n"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="92" t="inlineStr">
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="22" t="n"/>
+      <c r="F36" s="22" t="n"/>
+      <c r="G36" s="22" t="n"/>
+      <c r="H36" s="22" t="n"/>
+      <c r="I36" s="22" t="n"/>
+      <c r="J36" s="23" t="n"/>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="22" t="n"/>
+      <c r="O36" s="22" t="n"/>
+      <c r="P36" s="22" t="n"/>
+      <c r="Q36" s="23" t="n"/>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="11" t="n"/>
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="C36" s="93" t="inlineStr">
+      <c r="C37" s="26" t="inlineStr">
         <is>
           <t>Verificación de uniformidad de calor en todos los rodillos</t>
         </is>
       </c>
-      <c r="D36" s="100" t="n"/>
-      <c r="E36" s="100" t="n"/>
-      <c r="F36" s="100" t="n"/>
-      <c r="G36" s="100" t="n"/>
-      <c r="H36" s="100" t="n"/>
-      <c r="I36" s="100" t="n"/>
-      <c r="J36" s="101" t="n"/>
-      <c r="K36" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L36" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M36" s="95" t="n"/>
-      <c r="N36" s="101" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="B37" s="96" t="inlineStr">
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="22" t="n"/>
+      <c r="F37" s="22" t="n"/>
+      <c r="G37" s="22" t="n"/>
+      <c r="H37" s="22" t="n"/>
+      <c r="I37" s="22" t="n"/>
+      <c r="J37" s="23" t="n"/>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M37" s="51" t="n"/>
+      <c r="N37" s="50" t="n"/>
+      <c r="O37" s="50" t="n"/>
+      <c r="P37" s="50" t="n"/>
+      <c r="Q37" s="51" t="n"/>
+    </row>
+    <row r="38" ht="14.4" customHeight="1">
+      <c r="B38" s="24" t="inlineStr">
         <is>
           <t>CALENDARIO  DE  MANTENIMIENTO</t>
         </is>
       </c>
-      <c r="N37" s="102" t="inlineStr">
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
+      <c r="F38" s="22" t="n"/>
+      <c r="G38" s="22" t="n"/>
+      <c r="H38" s="22" t="n"/>
+      <c r="I38" s="22" t="n"/>
+      <c r="J38" s="22" t="n"/>
+      <c r="K38" s="22" t="n"/>
+      <c r="L38" s="22" t="n"/>
+      <c r="M38" s="23" t="n"/>
+      <c r="N38" s="43" t="inlineStr">
         <is>
           <t>VOLTAJE ALIMENTACIÓN</t>
         </is>
       </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="97" t="inlineStr">
+      <c r="O38" s="22" t="n"/>
+      <c r="P38" s="22" t="n"/>
+      <c r="Q38" s="23" t="n"/>
+    </row>
+    <row r="39" ht="14.4" customHeight="1">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>ENE</t>
         </is>
       </c>
-      <c r="C38" s="97" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="D38" s="97" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="E38" s="97" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>ABR</t>
         </is>
       </c>
-      <c r="F38" s="97" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="G38" s="97" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="H38" s="97" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="I38" s="97" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>AGO</t>
         </is>
       </c>
-      <c r="J38" s="97" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>SEP</t>
         </is>
       </c>
-      <c r="K38" s="97" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="L38" s="97" t="inlineStr">
+      <c r="L39" s="5" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="M38" s="97" t="inlineStr">
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>DIC</t>
         </is>
       </c>
-      <c r="N38" s="103" t="inlineStr">
+      <c r="N39" s="6" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
       </c>
-      <c r="O38" s="103" t="inlineStr">
+      <c r="O39" s="6" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
       </c>
-      <c r="P38" s="103" t="inlineStr">
+      <c r="P39" s="6" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
       </c>
-      <c r="Q38" s="103" t="inlineStr">
+      <c r="Q39" s="6" t="inlineStr">
         <is>
           <t>Fuente 24VDC
 (20-25 V)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="C39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="D39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="E39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="F39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="G39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="H39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="I39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="J39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="K39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M39" s="94" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="N39" s="104" t="n"/>
-      <c r="O39" s="104" t="n"/>
-      <c r="P39" s="104" t="n"/>
-      <c r="Q39" s="104" t="n"/>
-    </row>
-    <row r="41" ht="50" customHeight="1">
-      <c r="B41" s="85" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="n"/>
+      <c r="B41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Realizo: </t>
         </is>
       </c>
-      <c r="H41" s="98" t="inlineStr">
+      <c r="C41" s="50" t="n"/>
+      <c r="D41" s="50" t="n"/>
+      <c r="E41" s="50" t="n"/>
+      <c r="F41" s="50" t="n"/>
+      <c r="G41" s="51" t="n"/>
+      <c r="H41" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>
       </c>
-      <c r="J41" s="99" t="inlineStr">
+      <c r="I41" s="75" t="n"/>
+      <c r="J41" s="75" t="n"/>
+      <c r="K41" s="40" t="inlineStr">
         <is>
           <t>Supervisor de Mantenimiento:
 Firma: _____________________________</t>
         </is>
       </c>
+      <c r="L41" s="50" t="n"/>
+      <c r="M41" s="50" t="n"/>
+      <c r="N41" s="50" t="n"/>
+      <c r="O41" s="50" t="n"/>
+      <c r="P41" s="50" t="n"/>
+      <c r="Q41" s="51" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="98" t="inlineStr">
+      <c r="B42" s="39" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
+      <c r="C42" s="50" t="n"/>
+      <c r="D42" s="50" t="n"/>
+      <c r="E42" s="50" t="n"/>
+      <c r="F42" s="50" t="n"/>
+      <c r="G42" s="51" t="n"/>
+      <c r="K42" s="39" t="inlineStr">
+        <is>
+          <t>Firma:</t>
+        </is>
+      </c>
+      <c r="L42" s="50" t="n"/>
+      <c r="M42" s="50" t="n"/>
+      <c r="N42" s="50" t="n"/>
+      <c r="O42" s="50" t="n"/>
+      <c r="P42" s="50" t="n"/>
+      <c r="Q42" s="51" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="76">
+  <mergeCells count="80">
+    <mergeCell ref="M34:Q34"/>
+    <mergeCell ref="C30:J30"/>
+    <mergeCell ref="C33:J33"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="C35:J35"/>
+    <mergeCell ref="M35:Q35"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="J6:Q6"/>
+    <mergeCell ref="C25:J25"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="M30:Q30"/>
+    <mergeCell ref="M21:Q21"/>
+    <mergeCell ref="C11:J11"/>
+    <mergeCell ref="M33:Q33"/>
+    <mergeCell ref="M28:Q28"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="M27:Q27"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="K41:Q41"/>
+    <mergeCell ref="M24:Q24"/>
+    <mergeCell ref="C32:J32"/>
+    <mergeCell ref="M32:Q32"/>
+    <mergeCell ref="M14:Q14"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="N38:Q38"/>
     <mergeCell ref="C34:J34"/>
     <mergeCell ref="B42:G42"/>
-    <mergeCell ref="M34:N34"/>
     <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C33:J33"/>
     <mergeCell ref="C24:J24"/>
+    <mergeCell ref="J5:Q5"/>
     <mergeCell ref="H41:I41"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="C14:J14"/>
-    <mergeCell ref="I3:N3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="C35:J35"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="B38:M38"/>
     <mergeCell ref="C26:J26"/>
-    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="M20:Q20"/>
     <mergeCell ref="C29:J29"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="I5:N5"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="B37:M37"/>
-    <mergeCell ref="C25:J25"/>
-    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="M11:Q11"/>
     <mergeCell ref="C10:J10"/>
-    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="C16:J16"/>
+    <mergeCell ref="E3:N3"/>
+    <mergeCell ref="M10:Q10"/>
     <mergeCell ref="C22:J22"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I4:N4"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="C31:J31"/>
-    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M22:Q22"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="M13:Q13"/>
+    <mergeCell ref="M31:Q31"/>
     <mergeCell ref="C9:J9"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="M16:Q16"/>
+    <mergeCell ref="J4:Q4"/>
     <mergeCell ref="C12:J12"/>
-    <mergeCell ref="N37:Q37"/>
     <mergeCell ref="C21:J21"/>
-    <mergeCell ref="C11:J11"/>
-    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M25:Q25"/>
+    <mergeCell ref="M15:Q15"/>
     <mergeCell ref="B41:G41"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M37:Q37"/>
     <mergeCell ref="C36:J36"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="J41:N41"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="B16:J16"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M36:Q36"/>
+    <mergeCell ref="M18:Q18"/>
     <mergeCell ref="C23:J23"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="C17:J17"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="C32:J32"/>
-    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="M26:Q26"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="M17:Q17"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="M29:Q29"/>
+    <mergeCell ref="M23:Q23"/>
+    <mergeCell ref="B31:J31"/>
     <mergeCell ref="C28:J28"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C37:J37"/>
+    <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="K42:Q42"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Calender K1 Easy: agregar texto AD-PACK y CONVERSION en encabezado
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -157,6 +157,18 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001b5e20"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001b5e20"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="17">
@@ -589,7 +601,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -840,6 +852,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11117,9 +11135,13 @@
       <c r="P2" s="50" t="n"/>
       <c r="Q2" s="51" t="n"/>
     </row>
-    <row r="3" ht="97.8" customHeight="1">
+    <row r="3" ht="50" customHeight="1">
       <c r="A3" s="11" t="n"/>
-      <c r="B3" s="36" t="n"/>
+      <c r="B3" s="105" t="inlineStr">
+        <is>
+          <t>AD-PACK</t>
+        </is>
+      </c>
       <c r="C3" s="22" t="n"/>
       <c r="D3" s="23" t="n"/>
       <c r="E3" s="38" t="inlineStr">
@@ -11136,7 +11158,12 @@
       <c r="L3" s="22" t="n"/>
       <c r="M3" s="22" t="n"/>
       <c r="N3" s="23" t="n"/>
-      <c r="O3" s="35" t="n"/>
+      <c r="O3" s="106" t="inlineStr">
+        <is>
+          <t>CONVERSIÓN
+by AD-PACK</t>
+        </is>
+      </c>
       <c r="P3" s="22" t="n"/>
       <c r="Q3" s="23" t="n"/>
     </row>
@@ -12529,81 +12556,81 @@
   </sheetData>
   <mergeCells count="80">
     <mergeCell ref="M34:Q34"/>
-    <mergeCell ref="C30:J30"/>
     <mergeCell ref="C33:J33"/>
-    <mergeCell ref="B17:J17"/>
-    <mergeCell ref="C14:J14"/>
     <mergeCell ref="C35:J35"/>
-    <mergeCell ref="M35:Q35"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="J6:Q6"/>
     <mergeCell ref="C25:J25"/>
     <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="M30:Q30"/>
     <mergeCell ref="M21:Q21"/>
     <mergeCell ref="C11:J11"/>
-    <mergeCell ref="M33:Q33"/>
-    <mergeCell ref="M28:Q28"/>
-    <mergeCell ref="C27:J27"/>
     <mergeCell ref="M27:Q27"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="C8:J8"/>
     <mergeCell ref="K41:Q41"/>
     <mergeCell ref="M24:Q24"/>
     <mergeCell ref="C32:J32"/>
-    <mergeCell ref="M32:Q32"/>
-    <mergeCell ref="M14:Q14"/>
     <mergeCell ref="B5:I5"/>
-    <mergeCell ref="C19:J19"/>
     <mergeCell ref="C13:J13"/>
     <mergeCell ref="N38:Q38"/>
-    <mergeCell ref="C34:J34"/>
-    <mergeCell ref="B42:G42"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C24:J24"/>
     <mergeCell ref="J5:Q5"/>
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="B38:M38"/>
     <mergeCell ref="C26:J26"/>
     <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="C29:J29"/>
     <mergeCell ref="M11:Q11"/>
     <mergeCell ref="C10:J10"/>
     <mergeCell ref="C16:J16"/>
-    <mergeCell ref="E3:N3"/>
-    <mergeCell ref="M10:Q10"/>
-    <mergeCell ref="C22:J22"/>
     <mergeCell ref="M22:Q22"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="M13:Q13"/>
     <mergeCell ref="M31:Q31"/>
     <mergeCell ref="C9:J9"/>
-    <mergeCell ref="M7:Q7"/>
-    <mergeCell ref="M16:Q16"/>
     <mergeCell ref="J4:Q4"/>
-    <mergeCell ref="C12:J12"/>
-    <mergeCell ref="C21:J21"/>
-    <mergeCell ref="M25:Q25"/>
     <mergeCell ref="M15:Q15"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="M37:Q37"/>
     <mergeCell ref="C36:J36"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="M26:Q26"/>
+    <mergeCell ref="M29:Q29"/>
+    <mergeCell ref="M23:Q23"/>
+    <mergeCell ref="C28:J28"/>
+    <mergeCell ref="C37:J37"/>
+    <mergeCell ref="C30:J30"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="M35:Q35"/>
+    <mergeCell ref="M30:Q30"/>
+    <mergeCell ref="M33:Q33"/>
+    <mergeCell ref="M28:Q28"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="M32:Q32"/>
+    <mergeCell ref="M14:Q14"/>
+    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C34:J34"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B38:M38"/>
+    <mergeCell ref="C29:J29"/>
+    <mergeCell ref="E3:N3"/>
+    <mergeCell ref="M10:Q10"/>
+    <mergeCell ref="C22:J22"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="M13:Q13"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="M16:Q16"/>
+    <mergeCell ref="C12:J12"/>
+    <mergeCell ref="C21:J21"/>
+    <mergeCell ref="M25:Q25"/>
     <mergeCell ref="M36:Q36"/>
     <mergeCell ref="M18:Q18"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="O3:Q3"/>
     <mergeCell ref="M8:Q8"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="M26:Q26"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="M17:Q17"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="M29:Q29"/>
-    <mergeCell ref="M23:Q23"/>
     <mergeCell ref="B31:J31"/>
-    <mergeCell ref="C28:J28"/>
-    <mergeCell ref="C37:J37"/>
     <mergeCell ref="M19:Q19"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="K42:Q42"/>

</xml_diff>

<commit_message>
Calender K1 Easy: fijar area impresion B1:Q42 landscape una sola pagina
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -17,7 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hojeadora Robust" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gapcutter" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Calender K1 Easy'!$B$1:$Q$42</definedName>
+  </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -7242,6 +7244,22 @@
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
     <col width="12.77734375" customWidth="1" min="2" max="17"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.8" customHeight="1"/>
@@ -11096,13 +11114,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:Q42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
     <col width="12.77734375" customWidth="1" min="2" max="17"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.8" customHeight="1"/>
@@ -12636,7 +12670,7 @@
     <mergeCell ref="K42:Q42"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Komatsu OBS45: actualizar checklist con componentes reales (HOWA, Fuji, HDS, Komatsu G7, KONAN)
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gapcutter" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Komatsu OBS45'!$B$1:$Q$36</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Calender K1 Easy'!$B$1:$Q$42</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -6002,7 +6003,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:Q45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
@@ -6019,18 +6020,6 @@
           <t>AD-PACK  —  ÁREA DE CONVERSIÓN</t>
         </is>
       </c>
-      <c r="C2" s="22" t="n"/>
-      <c r="D2" s="22" t="n"/>
-      <c r="E2" s="22" t="n"/>
-      <c r="F2" s="22" t="n"/>
-      <c r="G2" s="22" t="n"/>
-      <c r="H2" s="22" t="n"/>
-      <c r="I2" s="22" t="n"/>
-      <c r="J2" s="22" t="n"/>
-      <c r="K2" s="22" t="n"/>
-      <c r="L2" s="22" t="n"/>
-      <c r="M2" s="22" t="n"/>
-      <c r="N2" s="23" t="n"/>
       <c r="O2" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve"> No. de Documento             A9.I1.F2
@@ -6038,31 +6027,16 @@
  Fecha:                        08/06/2026</t>
         </is>
       </c>
-      <c r="P2" s="50" t="n"/>
-      <c r="Q2" s="51" t="n"/>
     </row>
     <row r="3" ht="97.8" customHeight="1">
       <c r="A3" s="11" t="n"/>
       <c r="B3" s="36" t="n"/>
-      <c r="C3" s="22" t="n"/>
-      <c r="D3" s="23" t="n"/>
       <c r="E3" s="38" t="inlineStr">
         <is>
           <t>MANTENIMIENTO PREVENTIVO   —   KOMATSU OBS45 – PRENSA OBDS</t>
         </is>
       </c>
-      <c r="F3" s="22" t="n"/>
-      <c r="G3" s="22" t="n"/>
-      <c r="H3" s="22" t="n"/>
-      <c r="I3" s="22" t="n"/>
-      <c r="J3" s="22" t="n"/>
-      <c r="K3" s="22" t="n"/>
-      <c r="L3" s="22" t="n"/>
-      <c r="M3" s="22" t="n"/>
-      <c r="N3" s="23" t="n"/>
       <c r="O3" s="35" t="n"/>
-      <c r="P3" s="22" t="n"/>
-      <c r="Q3" s="23" t="n"/>
     </row>
     <row r="4" ht="25.05" customHeight="1">
       <c r="A4" s="11" t="n"/>
@@ -6071,25 +6045,11 @@
           <t>Alcance: Equipos de Conversión – AD-PACK</t>
         </is>
       </c>
-      <c r="C4" s="22" t="n"/>
-      <c r="D4" s="22" t="n"/>
-      <c r="E4" s="22" t="n"/>
-      <c r="F4" s="22" t="n"/>
-      <c r="G4" s="22" t="n"/>
-      <c r="H4" s="22" t="n"/>
-      <c r="I4" s="23" t="n"/>
       <c r="J4" s="33" t="inlineStr">
         <is>
           <t>Autor: Mariano Leyva</t>
         </is>
       </c>
-      <c r="K4" s="22" t="n"/>
-      <c r="L4" s="22" t="n"/>
-      <c r="M4" s="22" t="n"/>
-      <c r="N4" s="22" t="n"/>
-      <c r="O4" s="22" t="n"/>
-      <c r="P4" s="22" t="n"/>
-      <c r="Q4" s="23" t="n"/>
     </row>
     <row r="5" ht="46.2" customHeight="1">
       <c r="A5" s="11" t="n"/>
@@ -6098,25 +6058,11 @@
           <t>Tipo de mantenimiento:  Preventivo</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n"/>
-      <c r="D5" s="22" t="n"/>
-      <c r="E5" s="22" t="n"/>
-      <c r="F5" s="22" t="n"/>
-      <c r="G5" s="22" t="n"/>
-      <c r="H5" s="22" t="n"/>
-      <c r="I5" s="23" t="n"/>
       <c r="J5" s="33" t="inlineStr">
         <is>
           <t>Indicaciones: Usar equipo de seguridad.</t>
         </is>
       </c>
-      <c r="K5" s="22" t="n"/>
-      <c r="L5" s="22" t="n"/>
-      <c r="M5" s="22" t="n"/>
-      <c r="N5" s="22" t="n"/>
-      <c r="O5" s="22" t="n"/>
-      <c r="P5" s="22" t="n"/>
-      <c r="Q5" s="23" t="n"/>
     </row>
     <row r="6" ht="25.05" customHeight="1">
       <c r="A6" s="11" t="n"/>
@@ -6125,31 +6071,17 @@
           <t>Nombre de máquina:  Komatsu OBS45</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="22" t="n"/>
-      <c r="F6" s="22" t="n"/>
-      <c r="G6" s="22" t="n"/>
-      <c r="H6" s="22" t="n"/>
-      <c r="I6" s="23" t="n"/>
       <c r="J6" s="33" t="inlineStr">
         <is>
           <t>Número de máquina:  KO01</t>
         </is>
       </c>
-      <c r="K6" s="22" t="n"/>
-      <c r="L6" s="22" t="n"/>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="22" t="n"/>
-      <c r="O6" s="22" t="n"/>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="23" t="n"/>
     </row>
     <row r="7" ht="25.05" customHeight="1">
       <c r="A7" s="11" t="n"/>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MECÁNICO / HIDRÁULICO</t>
+          <t xml:space="preserve">  MECÁNICO / LUBRICACIÓN</t>
         </is>
       </c>
       <c r="C7" s="22" t="n"/>
@@ -6172,7 +6104,7 @@
       </c>
       <c r="M7" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMENTARIOS </t>
+          <t>COMENTARIOS</t>
         </is>
       </c>
       <c r="N7" s="22" t="n"/>
@@ -6189,7 +6121,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>Inspección visual de estructura, cilindros y mangueras</t>
+          <t>Inspección visual de estructura: guías, columnas y tornillería</t>
         </is>
       </c>
       <c r="D8" s="22" t="n"/>
@@ -6217,14 +6149,14 @@
     </row>
     <row r="9" ht="25.05" customHeight="1">
       <c r="A9" s="11" t="n"/>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>Verificación de nivel y calidad del aceite hidráulico</t>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Verificación del nivel de aceite Clutch &amp; Brake (visor - zona verde)</t>
         </is>
       </c>
       <c r="D9" s="22" t="n"/>
@@ -6259,7 +6191,7 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>Revisión de cilindros hidráulicos (vástagos, sellos y fugas)</t>
+          <t>Verificación del nivel de aceite Gear Box (visor - zona verde)</t>
         </is>
       </c>
       <c r="D10" s="22" t="n"/>
@@ -6287,14 +6219,14 @@
     </row>
     <row r="11" ht="25.05" customHeight="1">
       <c r="A11" s="11" t="n"/>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>Limpieza de filtro de aceite hidráulico</t>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Revisión de bomba de lubricación automática HOWA SMD: nivel de depósito</t>
         </is>
       </c>
       <c r="D11" s="22" t="n"/>
@@ -6329,7 +6261,7 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>Revisión de bomba hidráulica (ruido, presión y temperatura)</t>
+          <t>Verificar caudal y ciclos del lubricador HOWA (ajuste de descarga SMD3/SMD6)</t>
         </is>
       </c>
       <c r="D12" s="22" t="n"/>
@@ -6357,14 +6289,14 @@
     </row>
     <row r="13" ht="25.05" customHeight="1">
       <c r="A13" s="11" t="n"/>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
-        <is>
-          <t>Verificación de válvulas de control y alivio de presión</t>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Lubricación manual de guías y columnas (puntos de engrase)</t>
         </is>
       </c>
       <c r="D13" s="22" t="n"/>
@@ -6427,14 +6359,14 @@
     </row>
     <row r="15" ht="25.05" customHeight="1">
       <c r="A15" s="11" t="n"/>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
-        <is>
-          <t>Lubricación de guías, columnas y mecanismos de cierre</t>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Verificación de tornillería y fijaciones estructurales</t>
         </is>
       </c>
       <c r="D15" s="22" t="n"/>
@@ -6469,7 +6401,7 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>Verificación de tornillería y fijaciones estructurales</t>
+          <t>Revisión del contador D.MAINT en panel Komatsu (reseteo si aplica)</t>
         </is>
       </c>
       <c r="D16" s="22" t="n"/>
@@ -6497,16 +6429,12 @@
     </row>
     <row r="17" ht="25.05" customHeight="1">
       <c r="A17" s="11" t="n"/>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C17" s="59" t="inlineStr">
-        <is>
-          <t>Cambio de aceite hidráulico (programado)</t>
-        </is>
-      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ELÉCTRICO</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n"/>
       <c r="D17" s="22" t="n"/>
       <c r="E17" s="22" t="n"/>
       <c r="F17" s="22" t="n"/>
@@ -6514,17 +6442,21 @@
       <c r="H17" s="22" t="n"/>
       <c r="I17" s="22" t="n"/>
       <c r="J17" s="23" t="n"/>
-      <c r="K17" s="62" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L17" s="62" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M17" s="62" t="n"/>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L17" s="27" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="M17" s="27" t="inlineStr">
+        <is>
+          <t>COMENTARIOS</t>
+        </is>
+      </c>
       <c r="N17" s="22" t="n"/>
       <c r="O17" s="22" t="n"/>
       <c r="P17" s="22" t="n"/>
@@ -6532,12 +6464,16 @@
     </row>
     <row r="18" ht="25.05" customHeight="1">
       <c r="A18" s="11" t="n"/>
-      <c r="B18" s="71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ELÉCTRICO</t>
-        </is>
-      </c>
-      <c r="C18" s="58" t="n"/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Verificación del panel Komatsu: HMI, alarmas e indicadores (T.COUNT, L.COUNT, D.MAINT)</t>
+        </is>
+      </c>
       <c r="D18" s="22" t="n"/>
       <c r="E18" s="22" t="n"/>
       <c r="F18" s="22" t="n"/>
@@ -6545,21 +6481,17 @@
       <c r="H18" s="22" t="n"/>
       <c r="I18" s="22" t="n"/>
       <c r="J18" s="23" t="n"/>
-      <c r="K18" s="1" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L18" s="27" t="inlineStr">
-        <is>
-          <t>NG</t>
-        </is>
-      </c>
-      <c r="M18" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">COMENTARIOS </t>
-        </is>
-      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M18" s="27" t="n"/>
       <c r="N18" s="22" t="n"/>
       <c r="O18" s="22" t="n"/>
       <c r="P18" s="22" t="n"/>
@@ -6567,14 +6499,14 @@
     </row>
     <row r="19" ht="25.05" customHeight="1">
       <c r="A19" s="11" t="n"/>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t>Verificación visual del tablero (alarmas e indicadores)</t>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Verificación del VFD Komatsu G7 (CIMR-G7A2371, 3.7kW): parámetros, fallas y temperatura</t>
         </is>
       </c>
       <c r="D19" s="22" t="n"/>
@@ -6609,7 +6541,7 @@
       </c>
       <c r="C20" s="26" t="inlineStr">
         <is>
-          <t>Limpieza de tableros eléctricos y revisión de cableado</t>
+          <t>Verificación del transformador HDS HTIB-Y7.5KEULB (7.5kVA, 460→220V): temperatura</t>
         </is>
       </c>
       <c r="D20" s="22" t="n"/>
@@ -6637,14 +6569,14 @@
     </row>
     <row r="21" ht="25.05" customHeight="1">
       <c r="A21" s="11" t="n"/>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="C21" s="25" t="inlineStr">
-        <is>
-          <t>Reapriete de terminales en tablero eléctrico</t>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Revisión del interruptor principal Fuji BW50RAGU-3P020 (20A, 3P): estado y operación</t>
         </is>
       </c>
       <c r="D21" s="22" t="n"/>
@@ -6679,7 +6611,7 @@
       </c>
       <c r="C22" s="26" t="inlineStr">
         <is>
-          <t>Verificación de fusibles, contactores y relés térmicos</t>
+          <t>Limpieza de tablero eléctrico y revisión de borneras (U1, X1, X2, U2, V1, Y1Y2, V2, W1, Z1Z2, W2)</t>
         </is>
       </c>
       <c r="D22" s="22" t="n"/>
@@ -6707,14 +6639,14 @@
     </row>
     <row r="23" ht="25.05" customHeight="1">
       <c r="A23" s="11" t="n"/>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C23" s="25" t="inlineStr">
-        <is>
-          <t>Revisión de motores (temperatura, ruido y vibración)</t>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Reapriete de terminales y conexiones eléctricas</t>
         </is>
       </c>
       <c r="D23" s="22" t="n"/>
@@ -6749,7 +6681,7 @@
       </c>
       <c r="C24" s="26" t="inlineStr">
         <is>
-          <t>Revisión de sensores de posición y finales de carrera</t>
+          <t>Verificación de sensores de posición y finales de carrera</t>
         </is>
       </c>
       <c r="D24" s="22" t="n"/>
@@ -6777,14 +6709,14 @@
     </row>
     <row r="25" ht="25.05" customHeight="1">
       <c r="A25" s="11" t="n"/>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C25" s="25" t="inlineStr">
-        <is>
-          <t>Revisión de dispositivos de seguridad y cortina óptica</t>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Revisión de dispositivos de seguridad: doble mando (TWO HAND) y cortina óptica (LIGHT GUARD)</t>
         </is>
       </c>
       <c r="D25" s="22" t="n"/>
@@ -6819,7 +6751,7 @@
       </c>
       <c r="C26" s="26" t="inlineStr">
         <is>
-          <t>Prueba funcional de paros de emergencia</t>
+          <t>Prueba funcional de paros de emergencia (EMG. STOP/FAULT)</t>
         </is>
       </c>
       <c r="D26" s="22" t="n"/>
@@ -6847,12 +6779,12 @@
     </row>
     <row r="27" ht="25.05" customHeight="1">
       <c r="A27" s="11" t="n"/>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="C27" s="25" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>Verificación de tierras físicas y continuidad</t>
         </is>
@@ -6882,14 +6814,12 @@
     </row>
     <row r="28" ht="25.05" customHeight="1">
       <c r="A28" s="11" t="n"/>
-      <c r="B28" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C28" s="26" t="inlineStr">
-        <is>
-          <t>Termografía de tableros y conexiones</t>
-        </is>
-      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NEUMÁTICO</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n"/>
       <c r="D28" s="22" t="n"/>
       <c r="E28" s="22" t="n"/>
       <c r="F28" s="22" t="n"/>
@@ -6897,17 +6827,21 @@
       <c r="H28" s="22" t="n"/>
       <c r="I28" s="22" t="n"/>
       <c r="J28" s="23" t="n"/>
-      <c r="K28" s="52" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L28" s="52" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M28" s="52" t="n"/>
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="L28" s="27" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="M28" s="27" t="inlineStr">
+        <is>
+          <t>COMENTARIOS</t>
+        </is>
+      </c>
       <c r="N28" s="22" t="n"/>
       <c r="O28" s="22" t="n"/>
       <c r="P28" s="22" t="n"/>
@@ -6915,320 +6849,395 @@
     </row>
     <row r="29" ht="25.05" customHeight="1">
       <c r="A29" s="11" t="n"/>
-      <c r="B29" s="24" t="inlineStr">
-        <is>
-          <t>CALENDARIO  DE  MANTENIMIENTO</t>
-        </is>
-      </c>
-      <c r="C29" s="22" t="n"/>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>Verificación de presión de trabajo y purga de condensados</t>
+        </is>
+      </c>
       <c r="D29" s="22" t="n"/>
       <c r="E29" s="22" t="n"/>
       <c r="F29" s="22" t="n"/>
       <c r="G29" s="22" t="n"/>
       <c r="H29" s="22" t="n"/>
       <c r="I29" s="22" t="n"/>
-      <c r="J29" s="22" t="n"/>
-      <c r="K29" s="22" t="n"/>
-      <c r="L29" s="22" t="n"/>
-      <c r="M29" s="23" t="n"/>
-      <c r="N29" s="43" t="inlineStr">
-        <is>
-          <t>VOLTAJE ALIMENTACIÓN</t>
-        </is>
-      </c>
-      <c r="O29" s="22" t="n"/>
-      <c r="P29" s="22" t="n"/>
-      <c r="Q29" s="23" t="n"/>
+      <c r="J29" s="23" t="n"/>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="25.05" customHeight="1">
       <c r="A30" s="11" t="n"/>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>ENE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>FEB</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>ABR</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>MAY</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>JUN</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>JUL</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>AGO</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>SEP</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>OCT</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="inlineStr">
-        <is>
-          <t>NOV</t>
-        </is>
-      </c>
-      <c r="M30" s="5" t="inlineStr">
-        <is>
-          <t>DIC</t>
-        </is>
-      </c>
-      <c r="N30" s="6" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="O30" s="6" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="P30" s="6" t="inlineStr">
-        <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="Q30" s="6" t="inlineStr">
-        <is>
-          <t>VAC</t>
-        </is>
-      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Revisión del regulador de presión KONAN D4-15A-NR (ajuste y funcionamiento)</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="22" t="n"/>
+      <c r="F30" s="22" t="n"/>
+      <c r="G30" s="22" t="n"/>
+      <c r="H30" s="22" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="22" t="n"/>
+      <c r="O30" s="22" t="n"/>
+      <c r="P30" s="22" t="n"/>
+      <c r="Q30" s="23" t="n"/>
     </row>
     <row r="31" ht="25.05" customHeight="1">
       <c r="A31" s="11" t="n"/>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>(   )</t>
-        </is>
-      </c>
-      <c r="N31" s="6" t="n"/>
-      <c r="O31" s="6" t="n"/>
-      <c r="P31" s="6" t="n"/>
-      <c r="Q31" s="6" t="n"/>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>Inspección de mangueras, racores y conexiones neumáticas</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="22" t="n"/>
+      <c r="G31" s="22" t="n"/>
+      <c r="H31" s="22" t="n"/>
+      <c r="I31" s="22" t="n"/>
+      <c r="J31" s="23" t="n"/>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="22" t="n"/>
+      <c r="O31" s="22" t="n"/>
+      <c r="P31" s="22" t="n"/>
+      <c r="Q31" s="23" t="n"/>
     </row>
     <row r="32" ht="25.05" customHeight="1">
       <c r="A32" s="11" t="n"/>
-      <c r="B32" s="39" t="inlineStr">
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>CALENDARIO  DE  MANTENIMIENTO</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="22" t="n"/>
+      <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="22" t="n"/>
+      <c r="K32" s="22" t="n"/>
+      <c r="L32" s="22" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="43" t="inlineStr">
+        <is>
+          <t>VOLTAJE ALIMENTACIÓN</t>
+        </is>
+      </c>
+      <c r="O32" s="22" t="n"/>
+      <c r="P32" s="22" t="n"/>
+      <c r="Q32" s="23" t="n"/>
+    </row>
+    <row r="33" ht="25.05" customHeight="1">
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>ENE</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>FEB</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>ABR</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>MAY</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>JUN</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>NOV</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>DIC</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="Q33" s="6" t="inlineStr">
+        <is>
+          <t>VAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24.6" customHeight="1">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>(   )</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="n"/>
+      <c r="B35" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Realizo: </t>
         </is>
       </c>
-      <c r="C32" s="50" t="n"/>
-      <c r="D32" s="50" t="n"/>
-      <c r="E32" s="50" t="n"/>
-      <c r="F32" s="50" t="n"/>
-      <c r="G32" s="51" t="n"/>
-      <c r="H32" s="41" t="inlineStr">
+      <c r="C35" s="50" t="n"/>
+      <c r="D35" s="50" t="n"/>
+      <c r="E35" s="50" t="n"/>
+      <c r="F35" s="50" t="n"/>
+      <c r="G35" s="51" t="n"/>
+      <c r="H35" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>
       </c>
-      <c r="I32" s="75" t="n"/>
-      <c r="J32" s="75" t="n"/>
-      <c r="K32" s="40" t="inlineStr">
+      <c r="I35" s="75" t="n"/>
+      <c r="J35" s="75" t="n"/>
+      <c r="K35" s="40" t="inlineStr">
         <is>
           <t>Supervisor de Producción: 
 Firma: _____________________________</t>
         </is>
       </c>
-      <c r="L32" s="50" t="n"/>
-      <c r="M32" s="50" t="n"/>
-      <c r="N32" s="50" t="n"/>
-      <c r="O32" s="50" t="n"/>
-      <c r="P32" s="50" t="n"/>
-      <c r="Q32" s="51" t="n"/>
-    </row>
-    <row r="33" ht="25.05" customHeight="1">
-      <c r="B33" s="39" t="inlineStr">
+      <c r="L35" s="50" t="n"/>
+      <c r="M35" s="50" t="n"/>
+      <c r="N35" s="50" t="n"/>
+      <c r="O35" s="50" t="n"/>
+      <c r="P35" s="50" t="n"/>
+      <c r="Q35" s="51" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="39" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
-      <c r="C33" s="76" t="n"/>
-      <c r="D33" s="76" t="n"/>
-      <c r="E33" s="76" t="n"/>
-      <c r="F33" s="76" t="n"/>
-      <c r="G33" s="77" t="n"/>
-      <c r="K33" s="39" t="inlineStr">
+      <c r="C36" s="50" t="n"/>
+      <c r="D36" s="50" t="n"/>
+      <c r="E36" s="50" t="n"/>
+      <c r="F36" s="50" t="n"/>
+      <c r="G36" s="51" t="n"/>
+      <c r="K36" s="39" t="inlineStr">
         <is>
           <t>Firma:</t>
         </is>
       </c>
-      <c r="L33" s="76" t="n"/>
-      <c r="M33" s="76" t="n"/>
-      <c r="N33" s="76" t="n"/>
-      <c r="O33" s="76" t="n"/>
-      <c r="P33" s="76" t="n"/>
-      <c r="Q33" s="77" t="n"/>
-    </row>
-    <row r="34" ht="24.6" customHeight="1">
-      <c r="B34" s="78" t="n"/>
-      <c r="C34" s="79" t="n"/>
-      <c r="D34" s="79" t="n"/>
-      <c r="E34" s="79" t="n"/>
-      <c r="F34" s="79" t="n"/>
-      <c r="G34" s="80" t="n"/>
-      <c r="K34" s="78" t="n"/>
-      <c r="L34" s="79" t="n"/>
-      <c r="M34" s="79" t="n"/>
-      <c r="N34" s="79" t="n"/>
-      <c r="O34" s="79" t="n"/>
-      <c r="P34" s="79" t="n"/>
-      <c r="Q34" s="80" t="n"/>
+      <c r="L36" s="50" t="n"/>
+      <c r="M36" s="50" t="n"/>
+      <c r="N36" s="50" t="n"/>
+      <c r="O36" s="50" t="n"/>
+      <c r="P36" s="50" t="n"/>
+      <c r="Q36" s="51" t="n"/>
     </row>
     <row r="45">
       <c r="J45" s="18" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="62">
-    <mergeCell ref="B33:G34"/>
+  <mergeCells count="57">
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="C30:J30"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="C25:J25"/>
+    <mergeCell ref="N32:Q32"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="M30:Q30"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="M21:Q21"/>
+    <mergeCell ref="K36:Q36"/>
+    <mergeCell ref="C11:J11"/>
+    <mergeCell ref="M28:Q28"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="M27:Q27"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="M24:Q24"/>
+    <mergeCell ref="M14:Q14"/>
+    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C24:J24"/>
-    <mergeCell ref="J5:Q5"/>
-    <mergeCell ref="K33:Q34"/>
-    <mergeCell ref="C14:J14"/>
     <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="B29:M29"/>
     <mergeCell ref="C26:J26"/>
     <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="H32:J34"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="J6:Q6"/>
+    <mergeCell ref="C29:J29"/>
     <mergeCell ref="M11:Q11"/>
-    <mergeCell ref="C25:J25"/>
     <mergeCell ref="C10:J10"/>
     <mergeCell ref="C16:J16"/>
-    <mergeCell ref="E3:N3"/>
     <mergeCell ref="M10:Q10"/>
     <mergeCell ref="C22:J22"/>
     <mergeCell ref="M22:Q22"/>
-    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="C31:J31"/>
     <mergeCell ref="M13:Q13"/>
+    <mergeCell ref="M31:Q31"/>
     <mergeCell ref="C9:J9"/>
     <mergeCell ref="M7:Q7"/>
     <mergeCell ref="M16:Q16"/>
-    <mergeCell ref="J4:Q4"/>
-    <mergeCell ref="M12:Q12"/>
     <mergeCell ref="C12:J12"/>
+    <mergeCell ref="C21:J21"/>
     <mergeCell ref="M25:Q25"/>
-    <mergeCell ref="C21:J21"/>
     <mergeCell ref="M15:Q15"/>
-    <mergeCell ref="M21:Q21"/>
-    <mergeCell ref="C11:J11"/>
-    <mergeCell ref="B32:G32"/>
-    <mergeCell ref="M28:Q28"/>
-    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B32:M32"/>
+    <mergeCell ref="K35:Q35"/>
     <mergeCell ref="M18:Q18"/>
-    <mergeCell ref="M27:Q27"/>
     <mergeCell ref="C23:J23"/>
-    <mergeCell ref="K32:Q32"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="B2:N2"/>
     <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="M26:Q26"/>
     <mergeCell ref="B7:J7"/>
-    <mergeCell ref="C17:J17"/>
-    <mergeCell ref="B3:D3"/>
     <mergeCell ref="M17:Q17"/>
-    <mergeCell ref="M26:Q26"/>
-    <mergeCell ref="M24:Q24"/>
-    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="M29:Q29"/>
     <mergeCell ref="M23:Q23"/>
-    <mergeCell ref="M14:Q14"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="C28:J28"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C19:J19"/>
     <mergeCell ref="M19:Q19"/>
-    <mergeCell ref="N29:Q29"/>
-    <mergeCell ref="B4:I4"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Komatsu OBS45: aplicar alturas de fila y anchos de columna del formato Rotary Press
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -6010,6 +6010,22 @@
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
     <col width="12.77734375" customWidth="1" min="2" max="17"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.8" customHeight="1"/>
@@ -6028,7 +6044,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="97.8" customHeight="1">
+    <row r="3" ht="50" customHeight="1">
       <c r="A3" s="11" t="n"/>
       <c r="B3" s="36" t="n"/>
       <c r="E3" s="38" t="inlineStr">
@@ -6947,7 +6963,7 @@
       <c r="P31" s="22" t="n"/>
       <c r="Q31" s="23" t="n"/>
     </row>
-    <row r="32" ht="25.05" customHeight="1">
+    <row r="32" ht="17.4" customHeight="1">
       <c r="A32" s="11" t="n"/>
       <c r="B32" s="24" t="inlineStr">
         <is>
@@ -6974,7 +6990,7 @@
       <c r="P32" s="22" t="n"/>
       <c r="Q32" s="23" t="n"/>
     </row>
-    <row r="33" ht="25.05" customHeight="1">
+    <row r="33" ht="17.4" customHeight="1">
       <c r="B33" s="10" t="inlineStr">
         <is>
           <t>ENE</t>
@@ -7056,7 +7072,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="24.6" customHeight="1">
+    <row r="34" ht="17.4" customHeight="1">
       <c r="B34" s="9" t="inlineStr">
         <is>
           <t>(   )</t>
@@ -7118,7 +7134,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="24" customHeight="1">
       <c r="A35" s="11" t="n"/>
       <c r="B35" s="39" t="inlineStr">
         <is>
@@ -7150,7 +7166,7 @@
       <c r="P35" s="50" t="n"/>
       <c r="Q35" s="51" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="14.4" customHeight="1">
       <c r="B36" s="39" t="inlineStr">
         <is>
           <t>Firma:</t>
@@ -7180,38 +7196,24 @@
   <mergeCells count="57">
     <mergeCell ref="H35:I35"/>
     <mergeCell ref="C30:J30"/>
+    <mergeCell ref="C15:J15"/>
+    <mergeCell ref="C24:J24"/>
     <mergeCell ref="B17:J17"/>
     <mergeCell ref="C14:J14"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="B28:J28"/>
-    <mergeCell ref="C25:J25"/>
-    <mergeCell ref="N32:Q32"/>
-    <mergeCell ref="M12:Q12"/>
-    <mergeCell ref="M30:Q30"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="M21:Q21"/>
-    <mergeCell ref="K36:Q36"/>
-    <mergeCell ref="C11:J11"/>
-    <mergeCell ref="M28:Q28"/>
-    <mergeCell ref="C27:J27"/>
-    <mergeCell ref="M27:Q27"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="M24:Q24"/>
-    <mergeCell ref="M14:Q14"/>
-    <mergeCell ref="C19:J19"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C24:J24"/>
     <mergeCell ref="M9:Q9"/>
     <mergeCell ref="C26:J26"/>
     <mergeCell ref="M20:Q20"/>
     <mergeCell ref="C29:J29"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="B28:J28"/>
     <mergeCell ref="M11:Q11"/>
+    <mergeCell ref="C25:J25"/>
     <mergeCell ref="C10:J10"/>
     <mergeCell ref="C16:J16"/>
     <mergeCell ref="M10:Q10"/>
     <mergeCell ref="C22:J22"/>
     <mergeCell ref="M22:Q22"/>
+    <mergeCell ref="N32:Q32"/>
     <mergeCell ref="C31:J31"/>
     <mergeCell ref="M13:Q13"/>
     <mergeCell ref="M31:Q31"/>
@@ -7219,20 +7221,34 @@
     <mergeCell ref="M7:Q7"/>
     <mergeCell ref="M16:Q16"/>
     <mergeCell ref="C12:J12"/>
+    <mergeCell ref="M12:Q12"/>
+    <mergeCell ref="M30:Q30"/>
     <mergeCell ref="C21:J21"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="M21:Q21"/>
+    <mergeCell ref="K36:Q36"/>
     <mergeCell ref="M25:Q25"/>
+    <mergeCell ref="C11:J11"/>
     <mergeCell ref="M15:Q15"/>
     <mergeCell ref="B35:G35"/>
+    <mergeCell ref="M28:Q28"/>
     <mergeCell ref="B32:M32"/>
     <mergeCell ref="K35:Q35"/>
+    <mergeCell ref="C27:J27"/>
     <mergeCell ref="M18:Q18"/>
+    <mergeCell ref="M27:Q27"/>
     <mergeCell ref="C23:J23"/>
+    <mergeCell ref="C8:J8"/>
     <mergeCell ref="M8:Q8"/>
     <mergeCell ref="M26:Q26"/>
     <mergeCell ref="B7:J7"/>
     <mergeCell ref="M17:Q17"/>
+    <mergeCell ref="M24:Q24"/>
     <mergeCell ref="M29:Q29"/>
     <mergeCell ref="M23:Q23"/>
+    <mergeCell ref="M14:Q14"/>
+    <mergeCell ref="C19:J19"/>
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="M19:Q19"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fix Komatsu OBS45: agregar celdas combinadas en encabezado (filas 2-6) y corregir título
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -6005,7 +6005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:Q45"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -6036,6 +6036,18 @@
           <t>AD-PACK  —  ÁREA DE CONVERSIÓN</t>
         </is>
       </c>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="22" t="n"/>
+      <c r="F2" s="22" t="n"/>
+      <c r="G2" s="22" t="n"/>
+      <c r="H2" s="22" t="n"/>
+      <c r="I2" s="22" t="n"/>
+      <c r="J2" s="22" t="n"/>
+      <c r="K2" s="22" t="n"/>
+      <c r="L2" s="22" t="n"/>
+      <c r="M2" s="22" t="n"/>
+      <c r="N2" s="23" t="n"/>
       <c r="O2" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve"> No. de Documento             A9.I1.F2
@@ -6043,16 +6055,31 @@
  Fecha:                        08/06/2026</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="50" customHeight="1">
+      <c r="P2" s="50" t="n"/>
+      <c r="Q2" s="51" t="n"/>
+    </row>
+    <row r="3" ht="97.8" customHeight="1">
       <c r="A3" s="11" t="n"/>
       <c r="B3" s="36" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="23" t="n"/>
       <c r="E3" s="38" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO PREVENTIVO   —   KOMATSU OBS45 – PRENSA OBDS</t>
-        </is>
-      </c>
+          <t>MANTENIMIENTO PREVENTIVO   —   KOMATSU OBS45</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="n"/>
+      <c r="G3" s="22" t="n"/>
+      <c r="H3" s="22" t="n"/>
+      <c r="I3" s="22" t="n"/>
+      <c r="J3" s="22" t="n"/>
+      <c r="K3" s="22" t="n"/>
+      <c r="L3" s="22" t="n"/>
+      <c r="M3" s="22" t="n"/>
+      <c r="N3" s="23" t="n"/>
       <c r="O3" s="35" t="n"/>
+      <c r="P3" s="22" t="n"/>
+      <c r="Q3" s="23" t="n"/>
     </row>
     <row r="4" ht="25.05" customHeight="1">
       <c r="A4" s="11" t="n"/>
@@ -6061,11 +6088,25 @@
           <t>Alcance: Equipos de Conversión – AD-PACK</t>
         </is>
       </c>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="22" t="n"/>
+      <c r="H4" s="22" t="n"/>
+      <c r="I4" s="23" t="n"/>
       <c r="J4" s="33" t="inlineStr">
         <is>
           <t>Autor: Mariano Leyva</t>
         </is>
       </c>
+      <c r="K4" s="22" t="n"/>
+      <c r="L4" s="22" t="n"/>
+      <c r="M4" s="22" t="n"/>
+      <c r="N4" s="22" t="n"/>
+      <c r="O4" s="22" t="n"/>
+      <c r="P4" s="22" t="n"/>
+      <c r="Q4" s="23" t="n"/>
     </row>
     <row r="5" ht="46.2" customHeight="1">
       <c r="A5" s="11" t="n"/>
@@ -6074,24 +6115,52 @@
           <t>Tipo de mantenimiento:  Preventivo</t>
         </is>
       </c>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="22" t="n"/>
+      <c r="H5" s="22" t="n"/>
+      <c r="I5" s="23" t="n"/>
       <c r="J5" s="33" t="inlineStr">
         <is>
           <t>Indicaciones: Usar equipo de seguridad.</t>
         </is>
       </c>
+      <c r="K5" s="22" t="n"/>
+      <c r="L5" s="22" t="n"/>
+      <c r="M5" s="22" t="n"/>
+      <c r="N5" s="22" t="n"/>
+      <c r="O5" s="22" t="n"/>
+      <c r="P5" s="22" t="n"/>
+      <c r="Q5" s="23" t="n"/>
     </row>
     <row r="6" ht="25.05" customHeight="1">
       <c r="A6" s="11" t="n"/>
       <c r="B6" s="37" t="inlineStr">
         <is>
-          <t>Nombre de máquina:  Komatsu OBS45</t>
-        </is>
-      </c>
+          <t>Nombre de máquina:  Komatsu OBS45 – Prensa de Punzonado</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="22" t="n"/>
+      <c r="H6" s="22" t="n"/>
+      <c r="I6" s="23" t="n"/>
       <c r="J6" s="33" t="inlineStr">
         <is>
           <t>Número de máquina:  KO01</t>
         </is>
       </c>
+      <c r="K6" s="22" t="n"/>
+      <c r="L6" s="22" t="n"/>
+      <c r="M6" s="22" t="n"/>
+      <c r="N6" s="22" t="n"/>
+      <c r="O6" s="22" t="n"/>
+      <c r="P6" s="22" t="n"/>
+      <c r="Q6" s="23" t="n"/>
     </row>
     <row r="7" ht="25.05" customHeight="1">
       <c r="A7" s="11" t="n"/>
@@ -7193,11 +7262,12 @@
       <c r="J45" s="18" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
+  <mergeCells count="68">
     <mergeCell ref="H35:I35"/>
     <mergeCell ref="C30:J30"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C24:J24"/>
+    <mergeCell ref="J5:Q5"/>
     <mergeCell ref="B17:J17"/>
     <mergeCell ref="C14:J14"/>
     <mergeCell ref="M9:Q9"/>
@@ -7208,8 +7278,10 @@
     <mergeCell ref="B28:J28"/>
     <mergeCell ref="M11:Q11"/>
     <mergeCell ref="C25:J25"/>
+    <mergeCell ref="J6:Q6"/>
     <mergeCell ref="C10:J10"/>
     <mergeCell ref="C16:J16"/>
+    <mergeCell ref="E3:N3"/>
     <mergeCell ref="M10:Q10"/>
     <mergeCell ref="C22:J22"/>
     <mergeCell ref="M22:Q22"/>
@@ -7217,8 +7289,10 @@
     <mergeCell ref="C31:J31"/>
     <mergeCell ref="M13:Q13"/>
     <mergeCell ref="M31:Q31"/>
+    <mergeCell ref="O2:Q2"/>
     <mergeCell ref="C9:J9"/>
     <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="J4:Q4"/>
     <mergeCell ref="M16:Q16"/>
     <mergeCell ref="C12:J12"/>
     <mergeCell ref="M12:Q12"/>
@@ -7238,18 +7312,24 @@
     <mergeCell ref="M18:Q18"/>
     <mergeCell ref="M27:Q27"/>
     <mergeCell ref="C23:J23"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="O3:Q3"/>
     <mergeCell ref="C8:J8"/>
     <mergeCell ref="M8:Q8"/>
     <mergeCell ref="M26:Q26"/>
     <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B3:D3"/>
     <mergeCell ref="M17:Q17"/>
     <mergeCell ref="M24:Q24"/>
+    <mergeCell ref="B6:I6"/>
     <mergeCell ref="M29:Q29"/>
     <mergeCell ref="M23:Q23"/>
     <mergeCell ref="M14:Q14"/>
+    <mergeCell ref="B5:I5"/>
     <mergeCell ref="C19:J19"/>
     <mergeCell ref="C13:J13"/>
     <mergeCell ref="M19:Q19"/>
+    <mergeCell ref="B4:I4"/>
     <mergeCell ref="C18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7264,7 +7344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:Q39"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
Fix: celda Fecha verde centrada en Komatsu y Calender K1 Easy (expandir a H:J x 2 filas)
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -174,7 +174,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -262,6 +262,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002d8a45"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a5c2a"/>
       </patternFill>
     </fill>
   </fills>
@@ -604,7 +609,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -860,6 +865,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6005,7 +6013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q45"/>
+  <dimension ref="A2:Q45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -7215,7 +7223,7 @@
       <c r="E35" s="50" t="n"/>
       <c r="F35" s="50" t="n"/>
       <c r="G35" s="51" t="n"/>
-      <c r="H35" s="41" t="inlineStr">
+      <c r="H35" s="107" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>
@@ -7263,7 +7271,6 @@
     </row>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="H35:I35"/>
     <mergeCell ref="C30:J30"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C24:J24"/>
@@ -7283,6 +7290,7 @@
     <mergeCell ref="C16:J16"/>
     <mergeCell ref="E3:N3"/>
     <mergeCell ref="M10:Q10"/>
+    <mergeCell ref="H35:J36"/>
     <mergeCell ref="C22:J22"/>
     <mergeCell ref="M22:Q22"/>
     <mergeCell ref="N32:Q32"/>
@@ -7292,8 +7300,8 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="C9:J9"/>
     <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="M16:Q16"/>
     <mergeCell ref="J4:Q4"/>
-    <mergeCell ref="M16:Q16"/>
     <mergeCell ref="C12:J12"/>
     <mergeCell ref="M12:Q12"/>
     <mergeCell ref="M30:Q30"/>
@@ -7344,7 +7352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A2:Q39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -12649,7 +12657,7 @@
       <c r="E41" s="50" t="n"/>
       <c r="F41" s="50" t="n"/>
       <c r="G41" s="51" t="n"/>
-      <c r="H41" s="41" t="inlineStr">
+      <c r="H41" s="107" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>
@@ -12713,7 +12721,6 @@
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="C24:J24"/>
     <mergeCell ref="J5:Q5"/>
-    <mergeCell ref="H41:I41"/>
     <mergeCell ref="M9:Q9"/>
     <mergeCell ref="C26:J26"/>
     <mergeCell ref="M20:Q20"/>
@@ -12723,6 +12730,7 @@
     <mergeCell ref="M22:Q22"/>
     <mergeCell ref="M31:Q31"/>
     <mergeCell ref="C9:J9"/>
+    <mergeCell ref="H41:J42"/>
     <mergeCell ref="J4:Q4"/>
     <mergeCell ref="M15:Q15"/>
     <mergeCell ref="B41:G41"/>

</xml_diff>

<commit_message>
Fix: Komatsu sig_row 32→35, fgColor transparente→FF1A5C2A, template Fecha cells opaco
</commit_message>
<xml_diff>
--- a/MTTO_Preventivo_Conversion_2026.xlsx
+++ b/MTTO_Preventivo_Conversion_2026.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -173,8 +173,13 @@
       <color rgb="001b5e20"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -267,6 +272,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001a5c2a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A5C2A"/>
       </patternFill>
     </fill>
   </fills>
@@ -609,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -868,6 +878,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7223,7 +7236,7 @@
       <c r="E35" s="50" t="n"/>
       <c r="F35" s="50" t="n"/>
       <c r="G35" s="51" t="n"/>
-      <c r="H35" s="107" t="inlineStr">
+      <c r="H35" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>
@@ -12657,7 +12670,7 @@
       <c r="E41" s="50" t="n"/>
       <c r="F41" s="50" t="n"/>
       <c r="G41" s="51" t="n"/>
-      <c r="H41" s="107" t="inlineStr">
+      <c r="H41" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha: </t>
         </is>

</xml_diff>